<commit_message>
Add existing analyst click type labels from ADRIFT logs
</commit_message>
<xml_diff>
--- a/Analysis_Progress.xlsx
+++ b/Analysis_Progress.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9d4c4f1623d30376/Documents/GitHub/Rissos_Geographic_Variation/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\annes\Documents\Github\Rissos_Geographic_Variation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1888" documentId="8_{C4C2D1DD-6DD6-49C2-8C12-51DEE2FC981A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{65E9ED35-F36B-4BA0-B85D-1C793297B94E}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C61A8B44-91C0-44A5-AA70-9F2925166801}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="705" yWindow="705" windowWidth="16200" windowHeight="11025" activeTab="1" xr2:uid="{8391C37B-1672-4229-8478-45F991E75901}"/>
+    <workbookView xWindow="-35730" yWindow="2000" windowWidth="13680" windowHeight="18700" activeTab="1" xr2:uid="{8391C37B-1672-4229-8478-45F991E75901}"/>
   </bookViews>
   <sheets>
     <sheet name="Overall Progress" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1345" uniqueCount="270">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1367" uniqueCount="274">
   <si>
     <t>PG_Click_Detections</t>
   </si>
@@ -847,6 +847,18 @@
   </si>
   <si>
     <t>ADRIFT_068_005</t>
+  </si>
+  <si>
+    <t>Analyst Click Type Label</t>
+  </si>
+  <si>
+    <t>Ppac</t>
+  </si>
+  <si>
+    <t>CC</t>
+  </si>
+  <si>
+    <t>PPac</t>
   </si>
 </sst>
 </file>
@@ -1083,7 +1095,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="81">
+  <cellXfs count="84">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -1291,6 +1303,15 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1306,10 +1327,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1630,24 +1647,24 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3A18B98B-9FEB-4551-88CC-94F33BC1EF6E}">
   <dimension ref="A1:BR129"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18.46484375" style="51" customWidth="1"/>
-    <col min="2" max="2" width="18.46484375" style="14" customWidth="1"/>
-    <col min="3" max="3" width="19.06640625" style="14" customWidth="1"/>
-    <col min="4" max="4" width="29.19921875" style="14" customWidth="1"/>
-    <col min="5" max="5" width="23" style="14" customWidth="1"/>
-    <col min="6" max="10" width="24.1328125" style="14" customWidth="1"/>
-    <col min="11" max="11" width="47.53125" style="14" customWidth="1"/>
-    <col min="12" max="12" width="35.53125" style="14" customWidth="1"/>
-    <col min="13" max="13" width="50.73046875" style="2" customWidth="1"/>
-    <col min="14" max="14" width="38.86328125" style="2" customWidth="1"/>
+    <col min="1" max="1" width="18.42578125" style="51" customWidth="1"/>
+    <col min="2" max="2" width="18.42578125" style="14" customWidth="1"/>
+    <col min="3" max="3" width="19" style="14" customWidth="1"/>
+    <col min="4" max="4" width="29.140625" style="14" customWidth="1"/>
+    <col min="5" max="6" width="24.5703125" style="14" bestFit="1" customWidth="1"/>
+    <col min="7" max="10" width="24.140625" style="14" customWidth="1"/>
+    <col min="11" max="11" width="47.5703125" style="14" customWidth="1"/>
+    <col min="12" max="12" width="35.5703125" style="14" customWidth="1"/>
+    <col min="13" max="13" width="50.7109375" style="2" customWidth="1"/>
+    <col min="14" max="14" width="38.85546875" style="2" customWidth="1"/>
     <col min="15" max="15" width="53" style="2" customWidth="1"/>
-    <col min="16" max="16" width="9.06640625" style="13"/>
-    <col min="17" max="16384" width="9.06640625" style="14"/>
+    <col min="16" max="16" width="9" style="13"/>
+    <col min="17" max="16384" width="9" style="14"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:70" s="23" customFormat="1" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:70" s="23" customFormat="1" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="73" t="s">
         <v>3</v>
       </c>
@@ -1695,7 +1712,7 @@
       </c>
       <c r="P1" s="22"/>
     </row>
-    <row r="2" spans="1:70" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:70" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A2" s="51" t="s">
         <v>19</v>
       </c>
@@ -1733,7 +1750,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:70" s="24" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:70" s="24" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="74"/>
       <c r="B3" s="24" t="s">
         <v>63</v>
@@ -1821,7 +1838,7 @@
       <c r="BQ3" s="14"/>
       <c r="BR3" s="14"/>
     </row>
-    <row r="4" spans="1:70" s="11" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:70" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="64" t="s">
         <v>20</v>
       </c>
@@ -1919,7 +1936,7 @@
       <c r="BQ4" s="14"/>
       <c r="BR4" s="14"/>
     </row>
-    <row r="5" spans="1:70" s="11" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:70" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="64" t="s">
         <v>22</v>
       </c>
@@ -2015,7 +2032,7 @@
       <c r="BQ5" s="14"/>
       <c r="BR5" s="14"/>
     </row>
-    <row r="6" spans="1:70" s="26" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:70" s="26" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="51" t="s">
         <v>23</v>
       </c>
@@ -2059,7 +2076,7 @@
       </c>
       <c r="P6" s="28"/>
     </row>
-    <row r="7" spans="1:70" s="26" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:70" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="51"/>
       <c r="B7" s="26" t="s">
         <v>69</v>
@@ -2093,7 +2110,7 @@
       <c r="O7" s="8"/>
       <c r="P7" s="28"/>
     </row>
-    <row r="8" spans="1:70" s="26" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:70" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="51"/>
       <c r="B8" s="26" t="s">
         <v>70</v>
@@ -2127,7 +2144,7 @@
       <c r="O8" s="8"/>
       <c r="P8" s="28"/>
     </row>
-    <row r="9" spans="1:70" s="26" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:70" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="51"/>
       <c r="B9" s="26" t="s">
         <v>71</v>
@@ -2161,7 +2178,7 @@
       <c r="O9" s="8"/>
       <c r="P9" s="28"/>
     </row>
-    <row r="10" spans="1:70" s="29" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:70" s="29" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="74"/>
       <c r="B10" s="29" t="s">
         <v>72</v>
@@ -2249,7 +2266,7 @@
       <c r="BQ10" s="26"/>
       <c r="BR10" s="26"/>
     </row>
-    <row r="11" spans="1:70" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:70" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" s="54" t="s">
         <v>6</v>
       </c>
@@ -2293,7 +2310,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="12" spans="1:70" s="29" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:70" s="29" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="74"/>
       <c r="B12" s="29" t="s">
         <v>74</v>
@@ -2383,7 +2400,7 @@
       <c r="BQ12" s="26"/>
       <c r="BR12" s="26"/>
     </row>
-    <row r="13" spans="1:70" s="39" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:70" s="39" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="64" t="s">
         <v>8</v>
       </c>
@@ -2481,7 +2498,7 @@
       <c r="BQ13" s="26"/>
       <c r="BR13" s="26"/>
     </row>
-    <row r="14" spans="1:70" s="11" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:70" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="64" t="s">
         <v>9</v>
       </c>
@@ -2577,7 +2594,7 @@
       <c r="BQ14" s="14"/>
       <c r="BR14" s="14"/>
     </row>
-    <row r="15" spans="1:70" s="39" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:70" s="39" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" s="64" t="s">
         <v>25</v>
       </c>
@@ -2677,7 +2694,7 @@
       <c r="BQ15" s="26"/>
       <c r="BR15" s="26"/>
     </row>
-    <row r="16" spans="1:70" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:70" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="51" t="s">
         <v>26</v>
       </c>
@@ -2718,7 +2735,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="17" spans="1:70" s="29" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:70" s="29" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A17" s="74"/>
       <c r="B17" s="29" t="s">
         <v>79</v>
@@ -2810,7 +2827,7 @@
       <c r="BQ17" s="26"/>
       <c r="BR17" s="26"/>
     </row>
-    <row r="18" spans="1:70" s="39" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:70" s="39" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="64" t="s">
         <v>27</v>
       </c>
@@ -2908,7 +2925,7 @@
       <c r="BQ18" s="26"/>
       <c r="BR18" s="26"/>
     </row>
-    <row r="19" spans="1:70" s="11" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:70" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="64" t="s">
         <v>28</v>
       </c>
@@ -3004,7 +3021,7 @@
       <c r="BQ19" s="14"/>
       <c r="BR19" s="14"/>
     </row>
-    <row r="20" spans="1:70" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:70" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="51" t="s">
         <v>10</v>
       </c>
@@ -3051,7 +3068,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="21" spans="1:70" s="26" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:70" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="51"/>
       <c r="B21" s="26" t="s">
         <v>83</v>
@@ -3091,7 +3108,7 @@
       </c>
       <c r="P21" s="28"/>
     </row>
-    <row r="22" spans="1:70" s="26" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:70" s="26" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A22" s="51"/>
       <c r="B22" s="26" t="s">
         <v>84</v>
@@ -3128,7 +3145,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="23" spans="1:70" s="26" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:70" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="51"/>
       <c r="B23" s="26" t="s">
         <v>85</v>
@@ -3168,7 +3185,7 @@
       </c>
       <c r="P23" s="28"/>
     </row>
-    <row r="24" spans="1:70" s="29" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:70" s="29" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="74"/>
       <c r="B24" s="29" t="s">
         <v>86</v>
@@ -3260,7 +3277,7 @@
       <c r="BQ24" s="26"/>
       <c r="BR24" s="26"/>
     </row>
-    <row r="25" spans="1:70" s="26" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:70" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="51" t="s">
         <v>11</v>
       </c>
@@ -3306,7 +3323,7 @@
       </c>
       <c r="P25" s="28"/>
     </row>
-    <row r="26" spans="1:70" s="26" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:70" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="51"/>
       <c r="B26" s="26" t="s">
         <v>89</v>
@@ -3341,7 +3358,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="27" spans="1:70" s="26" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:70" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="51"/>
       <c r="B27" s="26" t="s">
         <v>88</v>
@@ -3376,7 +3393,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="28" spans="1:70" s="26" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:70" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="51"/>
       <c r="B28" s="26" t="s">
         <v>90</v>
@@ -3412,7 +3429,7 @@
       </c>
       <c r="P28" s="28"/>
     </row>
-    <row r="29" spans="1:70" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:70" x14ac:dyDescent="0.25">
       <c r="B29" s="14" t="s">
         <v>91</v>
       </c>
@@ -3441,7 +3458,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="30" spans="1:70" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:70" x14ac:dyDescent="0.25">
       <c r="B30" s="14" t="s">
         <v>92</v>
       </c>
@@ -3470,7 +3487,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="31" spans="1:70" s="24" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:70" s="24" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="74"/>
       <c r="B31" s="24" t="s">
         <v>253</v>
@@ -3558,7 +3575,7 @@
       <c r="BQ31" s="14"/>
       <c r="BR31" s="14"/>
     </row>
-    <row r="32" spans="1:70" s="26" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:70" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A32" s="51" t="s">
         <v>12</v>
       </c>
@@ -3604,7 +3621,7 @@
       </c>
       <c r="P32" s="28"/>
     </row>
-    <row r="33" spans="1:70" s="51" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:70" s="51" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B33" s="51" t="s">
         <v>94</v>
       </c>
@@ -3636,7 +3653,7 @@
       <c r="N33" s="54"/>
       <c r="P33" s="55"/>
     </row>
-    <row r="34" spans="1:70" s="29" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:70" s="29" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" s="74"/>
       <c r="B34" s="29" t="s">
         <v>95</v>
@@ -3728,7 +3745,7 @@
       <c r="BQ34" s="26"/>
       <c r="BR34" s="26"/>
     </row>
-    <row r="35" spans="1:70" s="39" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:70" s="39" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A35" s="64" t="s">
         <v>13</v>
       </c>
@@ -3826,7 +3843,7 @@
       <c r="BQ35" s="26"/>
       <c r="BR35" s="26"/>
     </row>
-    <row r="36" spans="1:70" x14ac:dyDescent="0.45">
+    <row r="36" spans="1:70" x14ac:dyDescent="0.25">
       <c r="A36" s="51" t="s">
         <v>14</v>
       </c>
@@ -3864,7 +3881,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="37" spans="1:70" s="29" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:70" s="29" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="74"/>
       <c r="B37" s="29" t="s">
         <v>98</v>
@@ -3954,7 +3971,7 @@
       <c r="BQ37" s="26"/>
       <c r="BR37" s="26"/>
     </row>
-    <row r="38" spans="1:70" x14ac:dyDescent="0.45">
+    <row r="38" spans="1:70" x14ac:dyDescent="0.25">
       <c r="A38" s="51" t="s">
         <v>15</v>
       </c>
@@ -3992,7 +4009,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="39" spans="1:70" x14ac:dyDescent="0.45">
+    <row r="39" spans="1:70" x14ac:dyDescent="0.25">
       <c r="B39" s="14" t="s">
         <v>100</v>
       </c>
@@ -4021,7 +4038,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="40" spans="1:70" x14ac:dyDescent="0.45">
+    <row r="40" spans="1:70" x14ac:dyDescent="0.25">
       <c r="B40" s="14" t="s">
         <v>101</v>
       </c>
@@ -4050,7 +4067,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="41" spans="1:70" x14ac:dyDescent="0.45">
+    <row r="41" spans="1:70" x14ac:dyDescent="0.25">
       <c r="B41" s="14" t="s">
         <v>102</v>
       </c>
@@ -4079,7 +4096,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="42" spans="1:70" s="24" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="42" spans="1:70" s="24" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A42" s="74"/>
       <c r="B42" s="24" t="s">
         <v>103</v>
@@ -4167,7 +4184,7 @@
       <c r="BQ42" s="14"/>
       <c r="BR42" s="14"/>
     </row>
-    <row r="43" spans="1:70" s="39" customFormat="1" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="43" spans="1:70" s="39" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A43" s="64" t="s">
         <v>29</v>
       </c>
@@ -4269,7 +4286,7 @@
       <c r="BQ43" s="26"/>
       <c r="BR43" s="26"/>
     </row>
-    <row r="44" spans="1:70" x14ac:dyDescent="0.45">
+    <row r="44" spans="1:70" x14ac:dyDescent="0.25">
       <c r="A44" s="51" t="s">
         <v>30</v>
       </c>
@@ -4307,7 +4324,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="45" spans="1:70" s="26" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="45" spans="1:70" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A45" s="51"/>
       <c r="B45" s="26" t="s">
         <v>107</v>
@@ -4343,7 +4360,7 @@
       </c>
       <c r="P45" s="28"/>
     </row>
-    <row r="46" spans="1:70" s="29" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="46" spans="1:70" s="29" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A46" s="74"/>
       <c r="B46" s="29" t="s">
         <v>113</v>
@@ -4431,7 +4448,7 @@
       <c r="BQ46" s="26"/>
       <c r="BR46" s="26"/>
     </row>
-    <row r="47" spans="1:70" s="11" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="47" spans="1:70" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A47" s="64" t="s">
         <v>31</v>
       </c>
@@ -4529,7 +4546,7 @@
       <c r="BQ47" s="14"/>
       <c r="BR47" s="14"/>
     </row>
-    <row r="48" spans="1:70" x14ac:dyDescent="0.45">
+    <row r="48" spans="1:70" x14ac:dyDescent="0.25">
       <c r="A48" s="51" t="s">
         <v>32</v>
       </c>
@@ -4573,7 +4590,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="49" spans="1:70" s="29" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="49" spans="1:70" s="29" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A49" s="74"/>
       <c r="B49" s="29" t="s">
         <v>255</v>
@@ -4663,7 +4680,7 @@
       <c r="BQ49" s="26"/>
       <c r="BR49" s="26"/>
     </row>
-    <row r="50" spans="1:70" s="11" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="50" spans="1:70" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A50" s="64" t="s">
         <v>33</v>
       </c>
@@ -4759,7 +4776,7 @@
       <c r="BQ50" s="14"/>
       <c r="BR50" s="14"/>
     </row>
-    <row r="51" spans="1:70" s="44" customFormat="1" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="51" spans="1:70" s="44" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A51" s="75" t="s">
         <v>34</v>
       </c>
@@ -4857,7 +4874,7 @@
       <c r="BQ51" s="26"/>
       <c r="BR51" s="26"/>
     </row>
-    <row r="52" spans="1:70" s="26" customFormat="1" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
+    <row r="52" spans="1:70" s="26" customFormat="1" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A52" s="51" t="s">
         <v>37</v>
       </c>
@@ -4901,7 +4918,7 @@
       </c>
       <c r="P52" s="28"/>
     </row>
-    <row r="53" spans="1:70" s="26" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="53" spans="1:70" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A53" s="51"/>
       <c r="B53" s="26" t="s">
         <v>114</v>
@@ -4935,7 +4952,7 @@
       <c r="O53" s="8"/>
       <c r="P53" s="28"/>
     </row>
-    <row r="54" spans="1:70" s="26" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="54" spans="1:70" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A54" s="51"/>
       <c r="B54" s="26" t="s">
         <v>115</v>
@@ -4969,7 +4986,7 @@
       <c r="O54" s="8"/>
       <c r="P54" s="28"/>
     </row>
-    <row r="55" spans="1:70" s="26" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="55" spans="1:70" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A55" s="51"/>
       <c r="B55" s="26" t="s">
         <v>116</v>
@@ -5003,7 +5020,7 @@
       <c r="O55" s="8"/>
       <c r="P55" s="28"/>
     </row>
-    <row r="56" spans="1:70" s="26" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="56" spans="1:70" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A56" s="51"/>
       <c r="B56" s="26" t="s">
         <v>117</v>
@@ -5037,7 +5054,7 @@
       <c r="O56" s="8"/>
       <c r="P56" s="28"/>
     </row>
-    <row r="57" spans="1:70" s="26" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="57" spans="1:70" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A57" s="51"/>
       <c r="B57" s="26" t="s">
         <v>66</v>
@@ -5071,7 +5088,7 @@
       <c r="O57" s="8"/>
       <c r="P57" s="28"/>
     </row>
-    <row r="58" spans="1:70" s="29" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="58" spans="1:70" s="29" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A58" s="74"/>
       <c r="B58" s="29" t="s">
         <v>118</v>
@@ -5159,7 +5176,7 @@
       <c r="BQ58" s="26"/>
       <c r="BR58" s="26"/>
     </row>
-    <row r="59" spans="1:70" s="26" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="59" spans="1:70" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A59" s="51" t="s">
         <v>36</v>
       </c>
@@ -5203,7 +5220,7 @@
       </c>
       <c r="P59" s="28"/>
     </row>
-    <row r="60" spans="1:70" s="26" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="60" spans="1:70" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A60" s="51"/>
       <c r="B60" s="26" t="s">
         <v>120</v>
@@ -5237,7 +5254,7 @@
       <c r="O60" s="8"/>
       <c r="P60" s="28"/>
     </row>
-    <row r="61" spans="1:70" s="26" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="61" spans="1:70" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A61" s="51"/>
       <c r="B61" s="26" t="s">
         <v>121</v>
@@ -5271,7 +5288,7 @@
       <c r="O61" s="8"/>
       <c r="P61" s="28"/>
     </row>
-    <row r="62" spans="1:70" s="26" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="62" spans="1:70" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A62" s="51"/>
       <c r="B62" s="26" t="s">
         <v>122</v>
@@ -5305,7 +5322,7 @@
       <c r="O62" s="8"/>
       <c r="P62" s="28"/>
     </row>
-    <row r="63" spans="1:70" s="29" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="63" spans="1:70" s="29" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A63" s="74"/>
       <c r="B63" s="29" t="s">
         <v>123</v>
@@ -5393,7 +5410,7 @@
       <c r="BQ63" s="26"/>
       <c r="BR63" s="26"/>
     </row>
-    <row r="64" spans="1:70" s="26" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="64" spans="1:70" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A64" s="51" t="s">
         <v>38</v>
       </c>
@@ -5439,7 +5456,7 @@
       </c>
       <c r="P64" s="28"/>
     </row>
-    <row r="65" spans="1:70" s="26" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="65" spans="1:70" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A65" s="51"/>
       <c r="B65" s="26" t="s">
         <v>125</v>
@@ -5477,7 +5494,7 @@
       </c>
       <c r="P65" s="28"/>
     </row>
-    <row r="66" spans="1:70" x14ac:dyDescent="0.45">
+    <row r="66" spans="1:70" x14ac:dyDescent="0.25">
       <c r="B66" s="14" t="s">
         <v>126</v>
       </c>
@@ -5509,7 +5526,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="67" spans="1:70" s="24" customFormat="1" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="67" spans="1:70" s="24" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A67" s="74"/>
       <c r="B67" s="24" t="s">
         <v>127</v>
@@ -5601,7 +5618,7 @@
       <c r="BQ67" s="14"/>
       <c r="BR67" s="14"/>
     </row>
-    <row r="68" spans="1:70" s="26" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="68" spans="1:70" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A68" s="51" t="s">
         <v>39</v>
       </c>
@@ -5645,7 +5662,7 @@
       </c>
       <c r="P68" s="28"/>
     </row>
-    <row r="69" spans="1:70" s="26" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="69" spans="1:70" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A69" s="51"/>
       <c r="B69" s="26" t="s">
         <v>129</v>
@@ -5679,7 +5696,7 @@
       <c r="O69" s="8"/>
       <c r="P69" s="28"/>
     </row>
-    <row r="70" spans="1:70" s="26" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="70" spans="1:70" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A70" s="51"/>
       <c r="B70" s="26" t="s">
         <v>130</v>
@@ -5713,7 +5730,7 @@
       <c r="O70" s="8"/>
       <c r="P70" s="28"/>
     </row>
-    <row r="71" spans="1:70" s="26" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="71" spans="1:70" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A71" s="51"/>
       <c r="B71" s="26" t="s">
         <v>131</v>
@@ -5747,7 +5764,7 @@
       <c r="O71" s="8"/>
       <c r="P71" s="28"/>
     </row>
-    <row r="72" spans="1:70" s="26" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="72" spans="1:70" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A72" s="51"/>
       <c r="B72" s="26" t="s">
         <v>132</v>
@@ -5781,7 +5798,7 @@
       <c r="O72" s="8"/>
       <c r="P72" s="28"/>
     </row>
-    <row r="73" spans="1:70" s="26" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="73" spans="1:70" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A73" s="51"/>
       <c r="B73" s="26" t="s">
         <v>133</v>
@@ -5815,7 +5832,7 @@
       <c r="O73" s="8"/>
       <c r="P73" s="28"/>
     </row>
-    <row r="74" spans="1:70" s="26" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="74" spans="1:70" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A74" s="51"/>
       <c r="B74" s="26" t="s">
         <v>134</v>
@@ -5849,7 +5866,7 @@
       <c r="O74" s="8"/>
       <c r="P74" s="28"/>
     </row>
-    <row r="75" spans="1:70" s="26" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="75" spans="1:70" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A75" s="51"/>
       <c r="B75" s="26" t="s">
         <v>135</v>
@@ -5883,7 +5900,7 @@
       <c r="O75" s="8"/>
       <c r="P75" s="28"/>
     </row>
-    <row r="76" spans="1:70" s="26" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="76" spans="1:70" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A76" s="51"/>
       <c r="B76" s="26" t="s">
         <v>136</v>
@@ -5917,7 +5934,7 @@
       <c r="O76" s="8"/>
       <c r="P76" s="28"/>
     </row>
-    <row r="77" spans="1:70" s="29" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="77" spans="1:70" s="29" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A77" s="74"/>
       <c r="B77" s="29" t="s">
         <v>137</v>
@@ -6005,7 +6022,7 @@
       <c r="BQ77" s="26"/>
       <c r="BR77" s="26"/>
     </row>
-    <row r="78" spans="1:70" s="26" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="78" spans="1:70" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A78" s="51" t="s">
         <v>35</v>
       </c>
@@ -6051,7 +6068,7 @@
       </c>
       <c r="P78" s="28"/>
     </row>
-    <row r="79" spans="1:70" s="33" customFormat="1" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="79" spans="1:70" s="33" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A79" s="76"/>
       <c r="B79" s="33" t="s">
         <v>139</v>
@@ -6141,7 +6158,7 @@
       <c r="BQ79" s="14"/>
       <c r="BR79" s="14"/>
     </row>
-    <row r="80" spans="1:70" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
+    <row r="80" spans="1:70" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A80" s="51" t="s">
         <v>40</v>
       </c>
@@ -6179,7 +6196,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="81" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="81" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B81" s="14" t="s">
         <v>141</v>
       </c>
@@ -6205,7 +6222,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="82" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="82" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B82" s="14" t="s">
         <v>142</v>
       </c>
@@ -6231,7 +6248,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="83" spans="1:16" s="24" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="83" spans="1:16" s="24" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A83" s="74"/>
       <c r="B83" s="24" t="s">
         <v>143</v>
@@ -6264,7 +6281,7 @@
       <c r="O83" s="5"/>
       <c r="P83" s="35"/>
     </row>
-    <row r="84" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="84" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A84" s="51" t="s">
         <v>41</v>
       </c>
@@ -6305,7 +6322,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="85" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="85" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B85" s="14" t="s">
         <v>145</v>
       </c>
@@ -6334,7 +6351,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="86" spans="1:16" s="26" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="86" spans="1:16" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A86" s="51"/>
       <c r="B86" s="26" t="s">
         <v>146</v>
@@ -6369,7 +6386,7 @@
       </c>
       <c r="P86" s="28"/>
     </row>
-    <row r="87" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="87" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B87" s="14" t="s">
         <v>147</v>
       </c>
@@ -6398,7 +6415,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="88" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="88" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B88" s="14" t="s">
         <v>148</v>
       </c>
@@ -6427,7 +6444,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="89" spans="1:16" s="26" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="89" spans="1:16" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A89" s="51"/>
       <c r="B89" s="26" t="s">
         <v>149</v>
@@ -6462,7 +6479,7 @@
       </c>
       <c r="P89" s="28"/>
     </row>
-    <row r="90" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="90" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B90" s="14" t="s">
         <v>150</v>
       </c>
@@ -6494,7 +6511,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="91" spans="1:16" s="26" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="91" spans="1:16" s="26" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A91" s="51"/>
       <c r="B91" s="26" t="s">
         <v>67</v>
@@ -6531,7 +6548,7 @@
       </c>
       <c r="P91" s="28"/>
     </row>
-    <row r="92" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="92" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B92" s="14" t="s">
         <v>151</v>
       </c>
@@ -6560,7 +6577,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="93" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="93" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B93" s="14" t="s">
         <v>152</v>
       </c>
@@ -6586,7 +6603,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="94" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="94" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B94" s="14" t="s">
         <v>153</v>
       </c>
@@ -6615,7 +6632,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="95" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="95" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B95" s="14" t="s">
         <v>154</v>
       </c>
@@ -6644,7 +6661,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="96" spans="1:16" s="26" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="96" spans="1:16" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A96" s="51"/>
       <c r="B96" s="26" t="s">
         <v>155</v>
@@ -6678,7 +6695,7 @@
       </c>
       <c r="P96" s="28"/>
     </row>
-    <row r="97" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="97" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B97" s="14" t="s">
         <v>156</v>
       </c>
@@ -6710,7 +6727,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="98" spans="1:16" s="26" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="98" spans="1:16" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A98" s="51"/>
       <c r="B98" s="26" t="s">
         <v>157</v>
@@ -6745,7 +6762,7 @@
       </c>
       <c r="P98" s="28"/>
     </row>
-    <row r="99" spans="1:16" s="26" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="99" spans="1:16" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A99" s="51"/>
       <c r="B99" s="26" t="s">
         <v>158</v>
@@ -6780,7 +6797,7 @@
       </c>
       <c r="P99" s="28"/>
     </row>
-    <row r="100" spans="1:16" s="26" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="100" spans="1:16" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A100" s="51"/>
       <c r="B100" s="26" t="s">
         <v>159</v>
@@ -6815,7 +6832,7 @@
       </c>
       <c r="P100" s="28"/>
     </row>
-    <row r="101" spans="1:16" s="26" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="101" spans="1:16" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A101" s="51"/>
       <c r="B101" s="26" t="s">
         <v>160</v>
@@ -6852,7 +6869,7 @@
       </c>
       <c r="P101" s="28"/>
     </row>
-    <row r="102" spans="1:16" s="26" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="102" spans="1:16" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A102" s="51"/>
       <c r="B102" s="26" t="s">
         <v>161</v>
@@ -6889,7 +6906,7 @@
       </c>
       <c r="P102" s="28"/>
     </row>
-    <row r="103" spans="1:16" s="26" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="103" spans="1:16" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A103" s="51"/>
       <c r="B103" s="26" t="s">
         <v>162</v>
@@ -6926,7 +6943,7 @@
       </c>
       <c r="P103" s="28"/>
     </row>
-    <row r="104" spans="1:16" s="26" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="104" spans="1:16" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A104" s="51"/>
       <c r="B104" s="26" t="s">
         <v>163</v>
@@ -6963,7 +6980,7 @@
       </c>
       <c r="P104" s="28"/>
     </row>
-    <row r="105" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="105" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B105" s="14" t="s">
         <v>164</v>
       </c>
@@ -6992,7 +7009,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="106" spans="1:16" s="26" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="106" spans="1:16" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A106" s="51"/>
       <c r="B106" s="26" t="s">
         <v>165</v>
@@ -7029,7 +7046,7 @@
       </c>
       <c r="P106" s="28"/>
     </row>
-    <row r="107" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="107" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B107" s="14" t="s">
         <v>166</v>
       </c>
@@ -7055,7 +7072,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="108" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="108" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B108" s="14" t="s">
         <v>167</v>
       </c>
@@ -7081,7 +7098,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="109" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="109" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B109" s="14" t="s">
         <v>168</v>
       </c>
@@ -7107,7 +7124,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="110" spans="1:16" s="26" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="110" spans="1:16" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A110" s="51"/>
       <c r="B110" s="26" t="s">
         <v>169</v>
@@ -7144,7 +7161,7 @@
       </c>
       <c r="P110" s="28"/>
     </row>
-    <row r="111" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="111" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B111" s="14" t="s">
         <v>170</v>
       </c>
@@ -7173,7 +7190,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="112" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="112" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B112" s="14" t="s">
         <v>171</v>
       </c>
@@ -7199,7 +7216,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="113" spans="1:16" s="26" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="113" spans="1:16" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A113" s="51"/>
       <c r="B113" s="26" t="s">
         <v>172</v>
@@ -7236,7 +7253,7 @@
       </c>
       <c r="P113" s="28"/>
     </row>
-    <row r="114" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="114" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B114" s="14" t="s">
         <v>173</v>
       </c>
@@ -7265,7 +7282,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="115" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="115" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B115" s="14" t="s">
         <v>174</v>
       </c>
@@ -7294,7 +7311,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="116" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="116" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B116" s="14" t="s">
         <v>175</v>
       </c>
@@ -7326,7 +7343,7 @@
         <v>251</v>
       </c>
     </row>
-    <row r="117" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="117" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B117" s="14" t="s">
         <v>176</v>
       </c>
@@ -7355,7 +7372,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="118" spans="1:16" s="26" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="118" spans="1:16" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A118" s="51"/>
       <c r="B118" s="26" t="s">
         <v>177</v>
@@ -7392,7 +7409,7 @@
       </c>
       <c r="P118" s="28"/>
     </row>
-    <row r="119" spans="1:16" s="26" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="119" spans="1:16" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A119" s="51"/>
       <c r="B119" s="26" t="s">
         <v>178</v>
@@ -7427,7 +7444,7 @@
       </c>
       <c r="P119" s="28"/>
     </row>
-    <row r="120" spans="1:16" s="26" customFormat="1" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="120" spans="1:16" s="26" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A120" s="51"/>
       <c r="B120" s="26" t="s">
         <v>179</v>
@@ -7464,7 +7481,7 @@
       </c>
       <c r="P120" s="28"/>
     </row>
-    <row r="121" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="121" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B121" s="14" t="s">
         <v>180</v>
       </c>
@@ -7496,7 +7513,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="122" spans="1:16" s="24" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="122" spans="1:16" s="24" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A122" s="74"/>
       <c r="B122" s="14" t="s">
         <v>181</v>
@@ -7531,7 +7548,7 @@
       <c r="O122" s="5"/>
       <c r="P122" s="35"/>
     </row>
-    <row r="123" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="123" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A123" s="64" t="s">
         <v>42</v>
       </c>
@@ -7572,7 +7589,7 @@
       <c r="O123" s="1"/>
       <c r="P123" s="36"/>
     </row>
-    <row r="124" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="124" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A124" s="51" t="s">
         <v>43</v>
       </c>
@@ -7607,7 +7624,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="125" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="125" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B125" s="14" t="s">
         <v>184</v>
       </c>
@@ -7633,7 +7650,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="126" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="126" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B126" s="14" t="s">
         <v>185</v>
       </c>
@@ -7662,7 +7679,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="127" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="127" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B127" s="14" t="s">
         <v>186</v>
       </c>
@@ -7691,7 +7708,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="128" spans="1:16" s="33" customFormat="1" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="128" spans="1:16" s="33" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A128" s="76"/>
       <c r="B128" s="33" t="s">
         <v>187</v>
@@ -7724,7 +7741,7 @@
       <c r="O128" s="19"/>
       <c r="P128" s="37"/>
     </row>
-    <row r="129" ht="14.65" thickTop="1" x14ac:dyDescent="0.45"/>
+    <row r="129" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -7735,15 +7752,17 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28DDFDEA-2838-4C23-95EB-05B925C7BB88}">
   <dimension ref="A1:F60"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.06640625" customWidth="1"/>
-    <col min="2" max="2" width="19.19921875" customWidth="1"/>
-    <col min="3" max="3" width="26.3984375" customWidth="1"/>
-    <col min="4" max="4" width="18.59765625" customWidth="1"/>
+    <col min="1" max="1" width="17" customWidth="1"/>
+    <col min="2" max="2" width="19.140625" customWidth="1"/>
+    <col min="3" max="3" width="26.42578125" customWidth="1"/>
+    <col min="4" max="4" width="18.5703125" customWidth="1"/>
+    <col min="5" max="5" width="52.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="30.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="20" t="s">
         <v>3</v>
       </c>
@@ -7756,8 +7775,11 @@
       <c r="D1" s="56" t="s">
         <v>256</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
+      <c r="F1" s="81" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A2" s="14" t="s">
         <v>19</v>
       </c>
@@ -7770,8 +7792,11 @@
       <c r="D2" s="57" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="F2" s="82" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="24"/>
       <c r="B3" s="24" t="s">
         <v>63</v>
@@ -7782,8 +7807,11 @@
       <c r="D3" s="58" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="F3" s="82" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="11" t="s">
         <v>20</v>
       </c>
@@ -7796,8 +7824,11 @@
       <c r="D4" s="58" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="F4" s="82" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="11" t="s">
         <v>22</v>
       </c>
@@ -7811,7 +7842,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>6</v>
       </c>
@@ -7824,8 +7855,11 @@
       <c r="D6" s="58" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" s="68" customFormat="1" x14ac:dyDescent="0.45">
+      <c r="F6" s="82" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" s="68" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
         <v>9</v>
       </c>
@@ -7839,8 +7873,11 @@
         <v>260</v>
       </c>
       <c r="E7"/>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="F7" s="82" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
         <v>26</v>
       </c>
@@ -7853,8 +7890,11 @@
       <c r="D8" s="61" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="F8" s="82" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="11" t="s">
         <v>28</v>
       </c>
@@ -7867,8 +7907,11 @@
       <c r="D9" s="61" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="F9" s="82" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="11" t="s">
         <v>10</v>
       </c>
@@ -7881,8 +7924,11 @@
       <c r="D10" s="61" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" s="68" customFormat="1" x14ac:dyDescent="0.45">
+      <c r="F10" s="82" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" s="68" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
         <v>11</v>
       </c>
@@ -7896,8 +7942,11 @@
         <v>260</v>
       </c>
       <c r="E11"/>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="F11" s="82" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="14"/>
       <c r="B12" s="26" t="s">
         <v>92</v>
@@ -7911,9 +7960,11 @@
       <c r="E12" s="68" t="s">
         <v>265</v>
       </c>
-      <c r="F12" s="68"/>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="F12" s="83" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="24"/>
       <c r="B13" s="24" t="s">
         <v>253</v>
@@ -7924,8 +7975,11 @@
       <c r="D13" s="58" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="F13" s="82" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="64" t="s">
         <v>12</v>
       </c>
@@ -7939,7 +7993,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="11" t="s">
         <v>14</v>
       </c>
@@ -7952,8 +8006,11 @@
       <c r="D15" s="61" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="F15" s="82" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="14" t="s">
         <v>15</v>
       </c>
@@ -7966,8 +8023,11 @@
       <c r="D16" s="57" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F16" s="82" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="14"/>
       <c r="B17" s="14" t="s">
         <v>100</v>
@@ -7978,8 +8038,11 @@
       <c r="D17" s="57" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F17" s="82" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="14"/>
       <c r="B18" s="14" t="s">
         <v>101</v>
@@ -7990,8 +8053,11 @@
       <c r="D18" s="57" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F18" s="82" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="14"/>
       <c r="B19" s="14" t="s">
         <v>102</v>
@@ -8002,8 +8068,11 @@
       <c r="D19" s="57" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F19" s="82" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="24"/>
       <c r="B20" s="24" t="s">
         <v>269</v>
@@ -8014,8 +8083,11 @@
       <c r="D20" s="58" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F20" s="82" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="14" t="s">
         <v>30</v>
       </c>
@@ -8028,8 +8100,11 @@
       <c r="D21" s="57" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="22" spans="1:5" s="68" customFormat="1" x14ac:dyDescent="0.45">
+      <c r="F21" s="82" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" s="68" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="11" t="s">
         <v>31</v>
       </c>
@@ -8043,8 +8118,11 @@
         <v>260</v>
       </c>
       <c r="E22"/>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F22" s="82" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="51" t="s">
         <v>32</v>
       </c>
@@ -8060,8 +8138,11 @@
       <c r="E23" s="68" t="s">
         <v>262</v>
       </c>
-    </row>
-    <row r="24" spans="1:5" s="68" customFormat="1" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="F23" s="83" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" s="68" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="59" t="s">
         <v>33</v>
       </c>
@@ -8075,8 +8156,11 @@
         <v>260</v>
       </c>
       <c r="E24"/>
-    </row>
-    <row r="25" spans="1:5" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
+      <c r="F24" s="82" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A25" s="14" t="s">
         <v>40</v>
       </c>
@@ -8091,7 +8175,7 @@
       </c>
       <c r="E25" s="69"/>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="14"/>
       <c r="B26" s="14" t="s">
         <v>141</v>
@@ -8103,7 +8187,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="14"/>
       <c r="B27" s="14" t="s">
         <v>142</v>
@@ -8115,7 +8199,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="28" spans="1:5" s="68" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:6" s="68" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="29"/>
       <c r="B28" s="29" t="s">
         <v>143</v>
@@ -8130,7 +8214,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="14" t="s">
         <v>41</v>
       </c>
@@ -8144,7 +8228,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" s="14"/>
       <c r="B30" s="14" t="s">
         <v>145</v>
@@ -8156,7 +8240,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="26"/>
       <c r="B31" s="14" t="s">
         <v>147</v>
@@ -8168,7 +8252,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" s="14"/>
       <c r="B32" s="14" t="s">
         <v>148</v>
@@ -8180,7 +8264,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="14"/>
       <c r="B33" s="14" t="s">
         <v>150</v>
@@ -8192,7 +8276,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="26"/>
       <c r="B34" s="14" t="s">
         <v>151</v>
@@ -8204,7 +8288,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="14"/>
       <c r="B35" s="14" t="s">
         <v>152</v>
@@ -8216,7 +8300,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="26"/>
       <c r="B36" s="14" t="s">
         <v>153</v>
@@ -8228,7 +8312,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="14"/>
       <c r="B37" s="14" t="s">
         <v>154</v>
@@ -8240,7 +8324,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="14"/>
       <c r="B38" s="14" t="s">
         <v>156</v>
@@ -8252,7 +8336,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="39" spans="1:5" s="68" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="39" spans="1:5" s="68" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A39" s="26"/>
       <c r="B39" s="26" t="s">
         <v>164</v>
@@ -8267,7 +8351,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" s="26"/>
       <c r="B40" s="14" t="s">
         <v>166</v>
@@ -8279,7 +8363,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" s="14"/>
       <c r="B41" s="14" t="s">
         <v>167</v>
@@ -8291,7 +8375,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" s="14"/>
       <c r="B42" s="14" t="s">
         <v>168</v>
@@ -8303,7 +8387,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" s="26"/>
       <c r="B43" s="14" t="s">
         <v>170</v>
@@ -8315,7 +8399,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" s="26"/>
       <c r="B44" s="14" t="s">
         <v>171</v>
@@ -8327,7 +8411,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" s="26"/>
       <c r="B45" s="14" t="s">
         <v>173</v>
@@ -8339,7 +8423,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" s="26"/>
       <c r="B46" s="14" t="s">
         <v>174</v>
@@ -8351,7 +8435,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="47" spans="1:5" s="68" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="47" spans="1:5" s="68" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A47" s="26"/>
       <c r="B47" s="26" t="s">
         <v>175</v>
@@ -8366,7 +8450,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" s="26"/>
       <c r="B48" s="14" t="s">
         <v>176</v>
@@ -8378,7 +8462,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="49" spans="1:5" s="68" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="49" spans="1:5" s="68" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A49" s="26"/>
       <c r="B49" s="26" t="s">
         <v>180</v>
@@ -8393,7 +8477,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="50" spans="1:5" s="68" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="50" spans="1:5" s="68" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A50" s="29"/>
       <c r="B50" s="29" t="s">
         <v>181</v>
@@ -8408,7 +8492,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="51" spans="1:5" s="69" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="51" spans="1:5" s="69" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A51" s="64" t="s">
         <v>42</v>
       </c>
@@ -8425,7 +8509,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" s="14" t="s">
         <v>43</v>
       </c>
@@ -8442,7 +8526,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" s="14"/>
       <c r="B53" s="14" t="s">
         <v>184</v>
@@ -8454,7 +8538,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" s="14"/>
       <c r="B54" s="14" t="s">
         <v>185</v>
@@ -8469,7 +8553,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" s="14"/>
       <c r="B55" s="26" t="s">
         <v>186</v>
@@ -8484,7 +8568,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="56" spans="1:5" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="56" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A56" s="60"/>
       <c r="B56" s="78" t="s">
         <v>187</v>
@@ -8499,7 +8583,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="57" spans="1:5" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
+    <row r="57" spans="1:5" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>38</v>
       </c>
@@ -8513,7 +8597,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58" s="63"/>
       <c r="B58" s="24" t="s">
         <v>127</v>
@@ -8528,7 +8612,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="59" spans="1:5" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="59" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A59" s="60" t="s">
         <v>35</v>
       </c>
@@ -8545,7 +8629,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="60" spans="1:5" ht="14.65" thickTop="1" x14ac:dyDescent="0.45"/>
+    <row r="60" spans="1:5" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
ICI and Min-Max Clustering
</commit_message>
<xml_diff>
--- a/Analysis_Progress.xlsx
+++ b/Analysis_Progress.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9d4c4f1623d30376/Documents/GitHub/Rissos_Geographic_Variation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="41" documentId="13_ncr:1_{C61A8B44-91C0-44A5-AA70-9F2925166801}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{77D18FFC-893B-4393-A821-9AF91D9ADD41}"/>
+  <xr:revisionPtr revIDLastSave="441" documentId="13_ncr:1_{C61A8B44-91C0-44A5-AA70-9F2925166801}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F3BFAC85-1BEF-4C2A-82D9-28B04014BC58}"/>
   <bookViews>
-    <workbookView xWindow="10718" yWindow="0" windowWidth="10965" windowHeight="12863" activeTab="1" xr2:uid="{8391C37B-1672-4229-8478-45F991E75901}"/>
+    <workbookView xWindow="10718" yWindow="0" windowWidth="10965" windowHeight="12863" firstSheet="1" activeTab="1" xr2:uid="{8391C37B-1672-4229-8478-45F991E75901}"/>
   </bookViews>
   <sheets>
     <sheet name="Overall Progress" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1388" uniqueCount="282">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1424" uniqueCount="306">
   <si>
     <t>PG_Click_Detections</t>
   </si>
@@ -882,7 +882,79 @@
     <t>Ppac? GoMx? CC? IHP?</t>
   </si>
   <si>
-    <t>***</t>
+    <t>Peak 1</t>
+  </si>
+  <si>
+    <t>Peak 2</t>
+  </si>
+  <si>
+    <t>Peak 3</t>
+  </si>
+  <si>
+    <t>Peak 4</t>
+  </si>
+  <si>
+    <t>Notch 1</t>
+  </si>
+  <si>
+    <t>Notch 2</t>
+  </si>
+  <si>
+    <t>Notch 3</t>
+  </si>
+  <si>
+    <t>Detection Start</t>
+  </si>
+  <si>
+    <t>Detection End</t>
+  </si>
+  <si>
+    <t>Notes (Based on LTSA)</t>
+  </si>
+  <si>
+    <t>Classification (PPac or CC)</t>
+  </si>
+  <si>
+    <t>Looks like 4th spectrogram in Soldevila 2017. 4th peak 6-7 kHz, 3rd notch 3-4 kHz lower - lines up better with GoMX</t>
+  </si>
+  <si>
+    <t>Looks like 4th spectrogram in Soldevila 2017. 4th peak 7-8 kHz, 3rd notch 4-5 kHz lower - lines up better with GoMX</t>
+  </si>
+  <si>
+    <t>Looks like 4th spectrogram in Soldevila 2017. 4th peak 7-8 kHz, 3rd notch 3-4 kHz lower - lines up better with GoMX</t>
+  </si>
+  <si>
+    <t>ADRIFT_055 needs to be interpolated to correct frequency grid</t>
+  </si>
+  <si>
+    <t>CCES_007 needs to be interpolated to correct frequency grid</t>
+  </si>
+  <si>
+    <t>CCES_008 needs to be interpolated to correct frequency grid</t>
+  </si>
+  <si>
+    <t>PASCAL_009 needs to be interpolated to correct frequency grid</t>
+  </si>
+  <si>
+    <t>CCES_013 needs to be interpolated to correct frequency grid</t>
+  </si>
+  <si>
+    <t>PASCAL_012 needs to be interpolated to correct frequency grid</t>
+  </si>
+  <si>
+    <t>Thoughts</t>
+  </si>
+  <si>
+    <t>Peak 5 (?)</t>
+  </si>
+  <si>
+    <t>Peak 6 (?)</t>
+  </si>
+  <si>
+    <t>Notch 4 (?)</t>
+  </si>
+  <si>
+    <t>Notch 5 (?)</t>
   </si>
 </sst>
 </file>
@@ -892,7 +964,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss\ \U\T\C"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -942,6 +1014,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="9" tint="-0.249977111117893"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -957,7 +1036,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="15">
+  <borders count="20">
     <border>
       <left/>
       <right/>
@@ -1115,11 +1194,72 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thick">
+        <color indexed="64"/>
+      </right>
+      <top style="thick">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thick">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thick">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thick">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thick">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thick">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thick">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="82">
+  <cellXfs count="130">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -1286,29 +1426,9 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -1321,14 +1441,212 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1687,7 +2005,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:70" s="23" customFormat="1" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A1" s="73" t="s">
+      <c r="A1" s="57" t="s">
         <v>3</v>
       </c>
       <c r="B1" s="20" t="s">
@@ -1773,7 +2091,7 @@
       </c>
     </row>
     <row r="3" spans="1:70" s="24" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="A3" s="74"/>
+      <c r="A3" s="58"/>
       <c r="B3" s="24" t="s">
         <v>63</v>
       </c>
@@ -1861,7 +2179,7 @@
       <c r="BR3" s="14"/>
     </row>
     <row r="4" spans="1:70" s="11" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="A4" s="64" t="s">
+      <c r="A4" s="56" t="s">
         <v>20</v>
       </c>
       <c r="B4" s="11" t="s">
@@ -1959,7 +2277,7 @@
       <c r="BR4" s="14"/>
     </row>
     <row r="5" spans="1:70" s="11" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="A5" s="64" t="s">
+      <c r="A5" s="56" t="s">
         <v>22</v>
       </c>
       <c r="B5" s="11" t="s">
@@ -2201,7 +2519,7 @@
       <c r="P9" s="28"/>
     </row>
     <row r="10" spans="1:70" s="29" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="A10" s="74"/>
+      <c r="A10" s="58"/>
       <c r="B10" s="29" t="s">
         <v>72</v>
       </c>
@@ -2333,7 +2651,7 @@
       </c>
     </row>
     <row r="12" spans="1:70" s="29" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="A12" s="74"/>
+      <c r="A12" s="58"/>
       <c r="B12" s="29" t="s">
         <v>74</v>
       </c>
@@ -2423,7 +2741,7 @@
       <c r="BR12" s="26"/>
     </row>
     <row r="13" spans="1:70" s="39" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="A13" s="64" t="s">
+      <c r="A13" s="56" t="s">
         <v>8</v>
       </c>
       <c r="B13" s="39" t="s">
@@ -2521,7 +2839,7 @@
       <c r="BR13" s="26"/>
     </row>
     <row r="14" spans="1:70" s="11" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="A14" s="64" t="s">
+      <c r="A14" s="56" t="s">
         <v>9</v>
       </c>
       <c r="B14" s="11" t="s">
@@ -2617,7 +2935,7 @@
       <c r="BR14" s="14"/>
     </row>
     <row r="15" spans="1:70" s="39" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="A15" s="64" t="s">
+      <c r="A15" s="56" t="s">
         <v>25</v>
       </c>
       <c r="B15" s="39" t="s">
@@ -2758,7 +3076,7 @@
       </c>
     </row>
     <row r="17" spans="1:70" s="29" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="A17" s="74"/>
+      <c r="A17" s="58"/>
       <c r="B17" s="29" t="s">
         <v>79</v>
       </c>
@@ -2850,7 +3168,7 @@
       <c r="BR17" s="26"/>
     </row>
     <row r="18" spans="1:70" s="39" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="A18" s="64" t="s">
+      <c r="A18" s="56" t="s">
         <v>27</v>
       </c>
       <c r="B18" s="39" t="s">
@@ -2948,7 +3266,7 @@
       <c r="BR18" s="26"/>
     </row>
     <row r="19" spans="1:70" s="11" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="A19" s="64" t="s">
+      <c r="A19" s="56" t="s">
         <v>28</v>
       </c>
       <c r="B19" s="11" t="s">
@@ -3208,7 +3526,7 @@
       <c r="P23" s="28"/>
     </row>
     <row r="24" spans="1:70" s="29" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="A24" s="74"/>
+      <c r="A24" s="58"/>
       <c r="B24" s="29" t="s">
         <v>86</v>
       </c>
@@ -3510,7 +3828,7 @@
       </c>
     </row>
     <row r="31" spans="1:70" s="24" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="A31" s="74"/>
+      <c r="A31" s="58"/>
       <c r="B31" s="24" t="s">
         <v>253</v>
       </c>
@@ -3676,7 +3994,7 @@
       <c r="P33" s="55"/>
     </row>
     <row r="34" spans="1:70" s="29" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="A34" s="74"/>
+      <c r="A34" s="58"/>
       <c r="B34" s="29" t="s">
         <v>95</v>
       </c>
@@ -3768,7 +4086,7 @@
       <c r="BR34" s="26"/>
     </row>
     <row r="35" spans="1:70" s="39" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="A35" s="64" t="s">
+      <c r="A35" s="56" t="s">
         <v>13</v>
       </c>
       <c r="B35" s="39" t="s">
@@ -3904,7 +4222,7 @@
       </c>
     </row>
     <row r="37" spans="1:70" s="29" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="A37" s="74"/>
+      <c r="A37" s="58"/>
       <c r="B37" s="29" t="s">
         <v>98</v>
       </c>
@@ -4119,7 +4437,7 @@
       </c>
     </row>
     <row r="42" spans="1:70" s="24" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="A42" s="74"/>
+      <c r="A42" s="58"/>
       <c r="B42" s="24" t="s">
         <v>103</v>
       </c>
@@ -4207,7 +4525,7 @@
       <c r="BR42" s="14"/>
     </row>
     <row r="43" spans="1:70" s="39" customFormat="1" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A43" s="64" t="s">
+      <c r="A43" s="56" t="s">
         <v>29</v>
       </c>
       <c r="B43" s="39" t="s">
@@ -4383,7 +4701,7 @@
       <c r="P45" s="28"/>
     </row>
     <row r="46" spans="1:70" s="29" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="A46" s="74"/>
+      <c r="A46" s="58"/>
       <c r="B46" s="29" t="s">
         <v>113</v>
       </c>
@@ -4471,7 +4789,7 @@
       <c r="BR46" s="26"/>
     </row>
     <row r="47" spans="1:70" s="11" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="A47" s="64" t="s">
+      <c r="A47" s="56" t="s">
         <v>31</v>
       </c>
       <c r="B47" s="11" t="s">
@@ -4487,7 +4805,7 @@
         <v>45122.301076388889</v>
       </c>
       <c r="F47" s="12">
-        <v>45122.310162037043</v>
+        <v>45122.310162037036</v>
       </c>
       <c r="G47" s="6" t="s">
         <v>7</v>
@@ -4613,7 +4931,7 @@
       </c>
     </row>
     <row r="49" spans="1:70" s="29" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="A49" s="74"/>
+      <c r="A49" s="58"/>
       <c r="B49" s="29" t="s">
         <v>255</v>
       </c>
@@ -4703,7 +5021,7 @@
       <c r="BR49" s="26"/>
     </row>
     <row r="50" spans="1:70" s="11" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="A50" s="64" t="s">
+      <c r="A50" s="56" t="s">
         <v>33</v>
       </c>
       <c r="B50" s="11" t="s">
@@ -4799,7 +5117,7 @@
       <c r="BR50" s="14"/>
     </row>
     <row r="51" spans="1:70" s="44" customFormat="1" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A51" s="75" t="s">
+      <c r="A51" s="59" t="s">
         <v>34</v>
       </c>
       <c r="B51" s="44" t="s">
@@ -5111,7 +5429,7 @@
       <c r="P57" s="28"/>
     </row>
     <row r="58" spans="1:70" s="29" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="A58" s="74"/>
+      <c r="A58" s="58"/>
       <c r="B58" s="29" t="s">
         <v>118</v>
       </c>
@@ -5345,7 +5663,7 @@
       <c r="P62" s="28"/>
     </row>
     <row r="63" spans="1:70" s="29" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="A63" s="74"/>
+      <c r="A63" s="58"/>
       <c r="B63" s="29" t="s">
         <v>123</v>
       </c>
@@ -5549,7 +5867,7 @@
       </c>
     </row>
     <row r="67" spans="1:70" s="24" customFormat="1" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A67" s="74"/>
+      <c r="A67" s="58"/>
       <c r="B67" s="24" t="s">
         <v>127</v>
       </c>
@@ -5957,7 +6275,7 @@
       <c r="P76" s="28"/>
     </row>
     <row r="77" spans="1:70" s="29" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="A77" s="74"/>
+      <c r="A77" s="58"/>
       <c r="B77" s="29" t="s">
         <v>137</v>
       </c>
@@ -6091,7 +6409,7 @@
       <c r="P78" s="28"/>
     </row>
     <row r="79" spans="1:70" s="33" customFormat="1" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A79" s="76"/>
+      <c r="A79" s="60"/>
       <c r="B79" s="33" t="s">
         <v>139</v>
       </c>
@@ -6271,7 +6589,7 @@
       </c>
     </row>
     <row r="83" spans="1:16" s="24" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="A83" s="74"/>
+      <c r="A83" s="58"/>
       <c r="B83" s="24" t="s">
         <v>143</v>
       </c>
@@ -7536,7 +7854,7 @@
       </c>
     </row>
     <row r="122" spans="1:16" s="24" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="A122" s="74"/>
+      <c r="A122" s="58"/>
       <c r="B122" s="14" t="s">
         <v>181</v>
       </c>
@@ -7571,7 +7889,7 @@
       <c r="P122" s="35"/>
     </row>
     <row r="123" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="A123" s="64" t="s">
+      <c r="A123" s="56" t="s">
         <v>42</v>
       </c>
       <c r="B123" s="11" t="s">
@@ -7731,7 +8049,7 @@
       </c>
     </row>
     <row r="128" spans="1:16" s="33" customFormat="1" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A128" s="76"/>
+      <c r="A128" s="60"/>
       <c r="B128" s="33" t="s">
         <v>187</v>
       </c>
@@ -7773,949 +8091,2461 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28DDFDEA-2838-4C23-95EB-05B925C7BB88}">
-  <dimension ref="A1:G60"/>
+  <dimension ref="A1:W60"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="17" customWidth="1"/>
-    <col min="2" max="2" width="19.1328125" customWidth="1"/>
-    <col min="3" max="3" width="26.3984375" customWidth="1"/>
-    <col min="4" max="4" width="18.59765625" customWidth="1"/>
-    <col min="5" max="5" width="52.73046875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="30.3984375" customWidth="1"/>
-    <col min="7" max="7" width="20.1328125" customWidth="1"/>
+    <col min="1" max="1" width="17" style="64" customWidth="1"/>
+    <col min="2" max="2" width="19.1328125" style="64" customWidth="1"/>
+    <col min="3" max="3" width="26.1328125" style="64" customWidth="1"/>
+    <col min="4" max="4" width="26.73046875" style="64" customWidth="1"/>
+    <col min="5" max="5" width="26.3984375" style="64" customWidth="1"/>
+    <col min="6" max="6" width="18.59765625" style="64" customWidth="1"/>
+    <col min="7" max="7" width="52.73046875" style="64" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="30.3984375" style="64" customWidth="1"/>
+    <col min="9" max="9" width="20.1328125" style="64" customWidth="1"/>
+    <col min="10" max="18" width="9.06640625" style="64"/>
+    <col min="19" max="21" width="9.6640625" style="64" customWidth="1"/>
+    <col min="22" max="22" width="10" style="64" customWidth="1"/>
+    <col min="23" max="23" width="90.19921875" style="64" customWidth="1"/>
+    <col min="24" max="16384" width="9.06640625" style="64"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A1" s="20" t="s">
+    <row r="1" spans="1:23" s="67" customFormat="1" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A1" s="65" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="20" t="s">
+      <c r="B1" s="65" t="s">
         <v>104</v>
       </c>
-      <c r="C1" s="20" t="s">
+      <c r="C1" s="65" t="s">
+        <v>288</v>
+      </c>
+      <c r="D1" s="65" t="s">
+        <v>289</v>
+      </c>
+      <c r="E1" s="65" t="s">
         <v>259</v>
       </c>
-      <c r="D1" s="56" t="s">
+      <c r="F1" s="66" t="s">
         <v>256</v>
       </c>
-      <c r="F1" s="81" t="s">
+      <c r="H1" s="116" t="s">
         <v>270</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="A2" s="14" t="s">
+      <c r="I1" s="117" t="s">
+        <v>301</v>
+      </c>
+      <c r="K1" s="118" t="s">
+        <v>281</v>
+      </c>
+      <c r="L1" s="119" t="s">
+        <v>282</v>
+      </c>
+      <c r="M1" s="119" t="s">
+        <v>283</v>
+      </c>
+      <c r="N1" s="119" t="s">
+        <v>284</v>
+      </c>
+      <c r="O1" s="119" t="s">
+        <v>302</v>
+      </c>
+      <c r="P1" s="119" t="s">
+        <v>303</v>
+      </c>
+      <c r="Q1" s="119" t="s">
+        <v>285</v>
+      </c>
+      <c r="R1" s="119" t="s">
+        <v>286</v>
+      </c>
+      <c r="S1" s="119" t="s">
+        <v>287</v>
+      </c>
+      <c r="T1" s="119" t="s">
+        <v>304</v>
+      </c>
+      <c r="U1" s="119" t="s">
+        <v>305</v>
+      </c>
+      <c r="V1" s="119" t="s">
+        <v>291</v>
+      </c>
+      <c r="W1" s="120" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="2" spans="1:23" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
+      <c r="A2" s="68" t="s">
         <v>19</v>
       </c>
-      <c r="B2" s="14" t="s">
+      <c r="B2" s="68" t="s">
         <v>62</v>
       </c>
-      <c r="C2" s="14" t="s">
+      <c r="C2" s="69">
+        <v>44403.170833333337</v>
+      </c>
+      <c r="D2" s="69">
+        <v>44403.179166666669</v>
+      </c>
+      <c r="E2" s="68" t="s">
         <v>258</v>
       </c>
-      <c r="D2" s="57" t="s">
+      <c r="F2" s="70" t="s">
         <v>260</v>
       </c>
-      <c r="F2" s="14" t="s">
+      <c r="H2" s="71" t="s">
         <v>271</v>
       </c>
-      <c r="G2" s="14" t="s">
+      <c r="I2" s="72" t="s">
         <v>274</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A3" s="24"/>
-      <c r="B3" s="24" t="s">
+      <c r="K2" s="73"/>
+      <c r="L2" s="61"/>
+      <c r="M2" s="61"/>
+      <c r="N2" s="61"/>
+      <c r="O2" s="61"/>
+      <c r="P2" s="61"/>
+      <c r="Q2" s="61"/>
+      <c r="R2" s="61"/>
+      <c r="S2" s="61"/>
+      <c r="T2" s="61"/>
+      <c r="U2" s="61"/>
+      <c r="V2" s="61"/>
+      <c r="W2" s="70"/>
+    </row>
+    <row r="3" spans="1:23" x14ac:dyDescent="0.45">
+      <c r="A3" s="74"/>
+      <c r="B3" s="74" t="s">
         <v>63</v>
       </c>
-      <c r="C3" s="24" t="s">
+      <c r="C3" s="75">
+        <v>44407.519768518519</v>
+      </c>
+      <c r="D3" s="75">
+        <v>44407.534814814819</v>
+      </c>
+      <c r="E3" s="74" t="s">
         <v>258</v>
       </c>
-      <c r="D3" s="58" t="s">
+      <c r="F3" s="76" t="s">
         <v>260</v>
       </c>
-      <c r="F3" s="14" t="s">
+      <c r="H3" s="71" t="s">
         <v>272</v>
       </c>
-      <c r="G3" s="14" t="s">
+      <c r="I3" s="72" t="s">
         <v>274</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A4" s="11" t="s">
+      <c r="K3" s="121"/>
+      <c r="L3" s="85"/>
+      <c r="M3" s="85"/>
+      <c r="N3" s="85"/>
+      <c r="O3" s="85"/>
+      <c r="P3" s="85"/>
+      <c r="Q3" s="85"/>
+      <c r="R3" s="85"/>
+      <c r="S3" s="85"/>
+      <c r="T3" s="85"/>
+      <c r="U3" s="85"/>
+      <c r="V3" s="85"/>
+      <c r="W3" s="76"/>
+    </row>
+    <row r="4" spans="1:23" x14ac:dyDescent="0.45">
+      <c r="A4" s="77" t="s">
         <v>20</v>
       </c>
-      <c r="B4" s="11" t="s">
+      <c r="B4" s="77" t="s">
         <v>64</v>
       </c>
-      <c r="C4" s="11" t="s">
+      <c r="C4" s="78">
+        <v>44404.561458333337</v>
+      </c>
+      <c r="D4" s="78">
+        <v>44404.602083333331</v>
+      </c>
+      <c r="E4" s="77" t="s">
         <v>257</v>
       </c>
-      <c r="D4" s="58" t="s">
+      <c r="F4" s="76" t="s">
         <v>260</v>
       </c>
-      <c r="F4" s="14" t="s">
+      <c r="H4" s="71" t="s">
         <v>273</v>
       </c>
-      <c r="G4" s="14" t="s">
+      <c r="I4" s="72" t="s">
         <v>274</v>
       </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A5" s="11" t="s">
+      <c r="K4" s="122"/>
+      <c r="L4" s="79"/>
+      <c r="M4" s="79"/>
+      <c r="N4" s="79"/>
+      <c r="O4" s="79"/>
+      <c r="P4" s="79"/>
+      <c r="Q4" s="79"/>
+      <c r="R4" s="79"/>
+      <c r="S4" s="79"/>
+      <c r="T4" s="79"/>
+      <c r="U4" s="79"/>
+      <c r="V4" s="79"/>
+      <c r="W4" s="80"/>
+    </row>
+    <row r="5" spans="1:23" x14ac:dyDescent="0.45">
+      <c r="A5" s="77" t="s">
         <v>22</v>
       </c>
-      <c r="B5" s="11" t="s">
+      <c r="B5" s="77" t="s">
         <v>65</v>
       </c>
-      <c r="C5" s="11" t="s">
+      <c r="C5" s="78">
+        <v>44360.256701388891</v>
+      </c>
+      <c r="D5" s="78">
+        <v>44360.28528935185</v>
+      </c>
+      <c r="E5" s="77" t="s">
         <v>258</v>
       </c>
-      <c r="D5" s="58" t="s">
+      <c r="F5" s="76" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A6" s="2" t="s">
+      <c r="H5" s="73"/>
+      <c r="I5" s="70"/>
+      <c r="K5" s="122"/>
+      <c r="L5" s="79"/>
+      <c r="M5" s="79"/>
+      <c r="N5" s="79"/>
+      <c r="O5" s="79"/>
+      <c r="P5" s="79"/>
+      <c r="Q5" s="79"/>
+      <c r="R5" s="79"/>
+      <c r="S5" s="79"/>
+      <c r="T5" s="79"/>
+      <c r="U5" s="79"/>
+      <c r="V5" s="79"/>
+      <c r="W5" s="80"/>
+    </row>
+    <row r="6" spans="1:23" x14ac:dyDescent="0.45">
+      <c r="A6" s="68" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="68" t="s">
         <v>73</v>
       </c>
-      <c r="C6" s="11" t="s">
+      <c r="C6" s="69">
+        <v>44735.246354166673</v>
+      </c>
+      <c r="D6" s="69">
+        <v>44735.249305555553</v>
+      </c>
+      <c r="E6" s="77" t="s">
         <v>258</v>
       </c>
-      <c r="D6" s="58" t="s">
+      <c r="F6" s="76" t="s">
         <v>260</v>
       </c>
-      <c r="F6" s="14" t="s">
+      <c r="H6" s="71" t="s">
         <v>271</v>
       </c>
-      <c r="G6" s="14" t="s">
+      <c r="I6" s="72" t="s">
         <v>276</v>
       </c>
-    </row>
-    <row r="7" spans="1:7" s="68" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="A7" s="11" t="s">
+      <c r="K6" s="122">
+        <v>22.1</v>
+      </c>
+      <c r="L6" s="79">
+        <v>24.9</v>
+      </c>
+      <c r="M6" s="79">
+        <v>29</v>
+      </c>
+      <c r="N6" s="79">
+        <v>32.9</v>
+      </c>
+      <c r="O6" s="79"/>
+      <c r="P6" s="79"/>
+      <c r="Q6" s="79">
+        <v>23.2</v>
+      </c>
+      <c r="R6" s="79">
+        <v>26.7</v>
+      </c>
+      <c r="S6" s="79">
+        <v>30.4</v>
+      </c>
+      <c r="T6" s="79"/>
+      <c r="U6" s="79"/>
+      <c r="V6" s="79" t="s">
+        <v>272</v>
+      </c>
+      <c r="W6" s="80" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="7" spans="1:23" s="82" customFormat="1" x14ac:dyDescent="0.45">
+      <c r="A7" s="77" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="11" t="s">
+      <c r="B7" s="77" t="s">
         <v>76</v>
       </c>
-      <c r="C7" s="62" t="s">
+      <c r="C7" s="78">
+        <v>44818.185706018507</v>
+      </c>
+      <c r="D7" s="78">
+        <v>44818.250856481478</v>
+      </c>
+      <c r="E7" s="79" t="s">
         <v>257</v>
       </c>
-      <c r="D7" s="61" t="s">
+      <c r="F7" s="80" t="s">
         <v>260</v>
       </c>
-      <c r="E7"/>
-      <c r="F7" s="14" t="s">
+      <c r="G7" s="64"/>
+      <c r="H7" s="71" t="s">
         <v>271</v>
       </c>
-      <c r="G7" s="69" t="s">
+      <c r="I7" s="81" t="s">
         <v>277</v>
       </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A8" s="14" t="s">
+      <c r="K7" s="123"/>
+      <c r="L7" s="100"/>
+      <c r="M7" s="100"/>
+      <c r="N7" s="100"/>
+      <c r="O7" s="100"/>
+      <c r="P7" s="100"/>
+      <c r="Q7" s="100"/>
+      <c r="R7" s="100"/>
+      <c r="S7" s="100"/>
+      <c r="T7" s="100"/>
+      <c r="U7" s="100"/>
+      <c r="V7" s="100"/>
+      <c r="W7" s="101"/>
+    </row>
+    <row r="8" spans="1:23" x14ac:dyDescent="0.45">
+      <c r="A8" s="68" t="s">
         <v>26</v>
       </c>
-      <c r="B8" s="14" t="s">
+      <c r="B8" s="68" t="s">
         <v>78</v>
       </c>
-      <c r="C8" s="62" t="s">
+      <c r="C8" s="69">
+        <v>44909.985347222217</v>
+      </c>
+      <c r="D8" s="69">
+        <v>44910.02342592593</v>
+      </c>
+      <c r="E8" s="79" t="s">
         <v>257</v>
       </c>
-      <c r="D8" s="61" t="s">
+      <c r="F8" s="80" t="s">
         <v>260</v>
       </c>
-      <c r="F8" s="14" t="s">
+      <c r="H8" s="71" t="s">
         <v>271</v>
       </c>
-      <c r="G8" s="14" t="s">
+      <c r="I8" s="72" t="s">
         <v>276</v>
       </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A9" s="11" t="s">
+      <c r="K8" s="122"/>
+      <c r="L8" s="79"/>
+      <c r="M8" s="79"/>
+      <c r="N8" s="79"/>
+      <c r="O8" s="79"/>
+      <c r="P8" s="79"/>
+      <c r="Q8" s="79"/>
+      <c r="R8" s="79"/>
+      <c r="S8" s="79"/>
+      <c r="T8" s="79"/>
+      <c r="U8" s="79"/>
+      <c r="V8" s="79"/>
+      <c r="W8" s="80"/>
+    </row>
+    <row r="9" spans="1:23" x14ac:dyDescent="0.45">
+      <c r="A9" s="77" t="s">
         <v>28</v>
       </c>
-      <c r="B9" s="11" t="s">
+      <c r="B9" s="77" t="s">
         <v>81</v>
       </c>
-      <c r="C9" s="63" t="s">
+      <c r="C9" s="78">
+        <v>45005.294664351852</v>
+      </c>
+      <c r="D9" s="78">
+        <v>45005.301898148136</v>
+      </c>
+      <c r="E9" s="85" t="s">
         <v>257</v>
       </c>
-      <c r="D9" s="61" t="s">
+      <c r="F9" s="80" t="s">
         <v>260</v>
       </c>
-      <c r="F9" s="14" t="s">
+      <c r="H9" s="71" t="s">
         <v>271</v>
       </c>
-      <c r="G9" s="14" t="s">
+      <c r="I9" s="72" t="s">
         <v>278</v>
       </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A10" s="11" t="s">
+      <c r="K9" s="122"/>
+      <c r="L9" s="79"/>
+      <c r="M9" s="79"/>
+      <c r="N9" s="79"/>
+      <c r="O9" s="79"/>
+      <c r="P9" s="79"/>
+      <c r="Q9" s="79"/>
+      <c r="R9" s="79"/>
+      <c r="S9" s="79"/>
+      <c r="T9" s="79"/>
+      <c r="U9" s="79"/>
+      <c r="V9" s="79"/>
+      <c r="W9" s="80"/>
+    </row>
+    <row r="10" spans="1:23" x14ac:dyDescent="0.45">
+      <c r="A10" s="77" t="s">
         <v>10</v>
       </c>
-      <c r="B10" s="11" t="s">
+      <c r="B10" s="77" t="s">
         <v>82</v>
       </c>
-      <c r="C10" s="62" t="s">
+      <c r="C10" s="78">
+        <v>45002.156157407408</v>
+      </c>
+      <c r="D10" s="78">
+        <v>45002.260150462957</v>
+      </c>
+      <c r="E10" s="79" t="s">
         <v>257</v>
       </c>
-      <c r="D10" s="61" t="s">
+      <c r="F10" s="80" t="s">
         <v>260</v>
       </c>
-      <c r="E10" t="s">
-        <v>281</v>
-      </c>
-      <c r="F10" s="14" t="s">
+      <c r="H10" s="71" t="s">
         <v>271</v>
       </c>
-      <c r="G10" s="14" t="s">
+      <c r="I10" s="72" t="s">
         <v>278</v>
       </c>
-    </row>
-    <row r="11" spans="1:7" s="68" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="A11" s="14" t="s">
+      <c r="K10" s="122">
+        <v>21.7</v>
+      </c>
+      <c r="L10" s="79">
+        <v>25.3</v>
+      </c>
+      <c r="M10" s="79">
+        <v>28.7</v>
+      </c>
+      <c r="N10" s="79">
+        <v>32.299999999999997</v>
+      </c>
+      <c r="O10" s="79"/>
+      <c r="P10" s="79"/>
+      <c r="Q10" s="79">
+        <v>23.4</v>
+      </c>
+      <c r="R10" s="79">
+        <v>26.9</v>
+      </c>
+      <c r="S10" s="79">
+        <v>30.5</v>
+      </c>
+      <c r="T10" s="79"/>
+      <c r="U10" s="79"/>
+      <c r="V10" s="79" t="s">
+        <v>272</v>
+      </c>
+      <c r="W10" s="80" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="11" spans="1:23" s="82" customFormat="1" x14ac:dyDescent="0.45">
+      <c r="A11" s="86" t="s">
         <v>11</v>
       </c>
-      <c r="B11" s="14" t="s">
+      <c r="B11" s="86" t="s">
         <v>91</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C11" s="87">
+        <v>45002.523240740753</v>
+      </c>
+      <c r="D11" s="87">
+        <v>45002.559004629627</v>
+      </c>
+      <c r="E11" s="88" t="s">
         <v>258</v>
       </c>
-      <c r="D11" s="57" t="s">
+      <c r="F11" s="81" t="s">
         <v>260</v>
       </c>
-      <c r="E11"/>
-      <c r="F11" s="14" t="s">
+      <c r="G11" s="89" t="s">
+        <v>295</v>
+      </c>
+      <c r="H11" s="71" t="s">
         <v>271</v>
       </c>
-      <c r="G11" s="69" t="s">
+      <c r="I11" s="81" t="s">
         <v>276</v>
       </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A12" s="14"/>
-      <c r="B12" s="26" t="s">
+      <c r="K11" s="83"/>
+      <c r="L11" s="62"/>
+      <c r="M11" s="62"/>
+      <c r="N11" s="62"/>
+      <c r="O11" s="62"/>
+      <c r="P11" s="62"/>
+      <c r="Q11" s="62"/>
+      <c r="R11" s="62"/>
+      <c r="S11" s="62"/>
+      <c r="T11" s="62"/>
+      <c r="U11" s="62"/>
+      <c r="V11" s="62"/>
+      <c r="W11" s="84"/>
+    </row>
+    <row r="12" spans="1:23" x14ac:dyDescent="0.45">
+      <c r="A12" s="86"/>
+      <c r="B12" s="90" t="s">
         <v>92</v>
       </c>
-      <c r="C12" s="68" t="s">
+      <c r="C12" s="91"/>
+      <c r="D12" s="91"/>
+      <c r="E12" s="82" t="s">
         <v>257</v>
       </c>
-      <c r="D12" s="72" t="s">
+      <c r="F12" s="84" t="s">
         <v>261</v>
       </c>
-      <c r="E12" s="68" t="s">
+      <c r="G12" s="82" t="s">
         <v>265</v>
       </c>
-      <c r="F12" s="26" t="s">
+      <c r="H12" s="92" t="s">
         <v>271</v>
       </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A13" s="24"/>
-      <c r="B13" s="24" t="s">
+      <c r="I12" s="70"/>
+      <c r="K12" s="73"/>
+      <c r="L12" s="61"/>
+      <c r="M12" s="61"/>
+      <c r="N12" s="61"/>
+      <c r="O12" s="61"/>
+      <c r="P12" s="61"/>
+      <c r="Q12" s="61"/>
+      <c r="R12" s="61"/>
+      <c r="S12" s="61"/>
+      <c r="T12" s="61"/>
+      <c r="U12" s="61"/>
+      <c r="V12" s="61"/>
+      <c r="W12" s="70"/>
+    </row>
+    <row r="13" spans="1:23" x14ac:dyDescent="0.45">
+      <c r="A13" s="93"/>
+      <c r="B13" s="93" t="s">
         <v>253</v>
       </c>
-      <c r="C13" s="63" t="s">
+      <c r="C13" s="94">
+        <v>45003.336469907408</v>
+      </c>
+      <c r="D13" s="94">
+        <v>45003.382997685178</v>
+      </c>
+      <c r="E13" s="95" t="s">
         <v>258</v>
       </c>
-      <c r="D13" s="58" t="s">
+      <c r="F13" s="96" t="s">
         <v>260</v>
       </c>
-      <c r="F13" s="14" t="s">
+      <c r="H13" s="71" t="s">
         <v>271</v>
       </c>
-      <c r="G13" s="14" t="s">
+      <c r="I13" s="72" t="s">
         <v>278</v>
       </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A14" s="64" t="s">
+      <c r="K13" s="121"/>
+      <c r="L13" s="85"/>
+      <c r="M13" s="85"/>
+      <c r="N13" s="85"/>
+      <c r="O13" s="85"/>
+      <c r="P13" s="85"/>
+      <c r="Q13" s="85"/>
+      <c r="R13" s="85"/>
+      <c r="S13" s="85"/>
+      <c r="T13" s="85"/>
+      <c r="U13" s="85"/>
+      <c r="V13" s="85"/>
+      <c r="W13" s="76"/>
+    </row>
+    <row r="14" spans="1:23" x14ac:dyDescent="0.45">
+      <c r="A14" s="97" t="s">
         <v>12</v>
       </c>
-      <c r="B14" s="64" t="s">
+      <c r="B14" s="97" t="s">
         <v>94</v>
       </c>
-      <c r="C14" s="62" t="s">
+      <c r="C14" s="98">
+        <v>45003.131979166668</v>
+      </c>
+      <c r="D14" s="98">
+        <v>45003.165717592587</v>
+      </c>
+      <c r="E14" s="79" t="s">
         <v>257</v>
       </c>
-      <c r="D14" s="61" t="s">
+      <c r="F14" s="80" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A15" s="11" t="s">
+      <c r="H14" s="73"/>
+      <c r="I14" s="70"/>
+      <c r="K14" s="122">
+        <v>21.8</v>
+      </c>
+      <c r="L14" s="79">
+        <v>25.1</v>
+      </c>
+      <c r="M14" s="79">
+        <v>28.9</v>
+      </c>
+      <c r="N14" s="79">
+        <v>32.4</v>
+      </c>
+      <c r="O14" s="79"/>
+      <c r="P14" s="79"/>
+      <c r="Q14" s="79">
+        <v>23.6</v>
+      </c>
+      <c r="R14" s="79">
+        <v>27.2</v>
+      </c>
+      <c r="S14" s="79">
+        <v>30.8</v>
+      </c>
+      <c r="T14" s="79"/>
+      <c r="U14" s="79"/>
+      <c r="V14" s="79" t="s">
+        <v>272</v>
+      </c>
+      <c r="W14" s="80" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="15" spans="1:23" x14ac:dyDescent="0.45">
+      <c r="A15" s="77" t="s">
         <v>14</v>
       </c>
-      <c r="B15" s="11" t="s">
+      <c r="B15" s="77" t="s">
         <v>97</v>
       </c>
-      <c r="C15" s="62" t="s">
+      <c r="C15" s="78">
+        <v>45054.301666666674</v>
+      </c>
+      <c r="D15" s="78">
+        <v>45054.370532407411</v>
+      </c>
+      <c r="E15" s="79" t="s">
         <v>258</v>
       </c>
-      <c r="D15" s="61" t="s">
+      <c r="F15" s="80" t="s">
         <v>260</v>
       </c>
-      <c r="F15" s="14" t="s">
+      <c r="H15" s="71" t="s">
         <v>271</v>
       </c>
-      <c r="G15" t="s">
+      <c r="I15" s="70" t="s">
         <v>275</v>
       </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A16" s="14" t="s">
+      <c r="K15" s="121"/>
+      <c r="L15" s="85"/>
+      <c r="M15" s="85"/>
+      <c r="N15" s="85"/>
+      <c r="O15" s="85"/>
+      <c r="P15" s="85"/>
+      <c r="Q15" s="85"/>
+      <c r="R15" s="85"/>
+      <c r="S15" s="85"/>
+      <c r="T15" s="85"/>
+      <c r="U15" s="85"/>
+      <c r="V15" s="85"/>
+      <c r="W15" s="76"/>
+    </row>
+    <row r="16" spans="1:23" x14ac:dyDescent="0.45">
+      <c r="A16" s="68" t="s">
         <v>15</v>
       </c>
-      <c r="B16" s="14" t="s">
+      <c r="B16" s="68" t="s">
         <v>99</v>
       </c>
-      <c r="C16" t="s">
+      <c r="C16" s="69">
+        <v>45054.290162037039</v>
+      </c>
+      <c r="D16" s="69">
+        <v>45054.302893518507</v>
+      </c>
+      <c r="E16" s="64" t="s">
         <v>258</v>
       </c>
-      <c r="D16" s="57" t="s">
+      <c r="F16" s="70" t="s">
         <v>260</v>
       </c>
-      <c r="F16" s="14" t="s">
+      <c r="H16" s="71" t="s">
         <v>271</v>
       </c>
-      <c r="G16" t="s">
+      <c r="I16" s="70" t="s">
         <v>279</v>
       </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A17" s="14"/>
-      <c r="B17" s="14" t="s">
+      <c r="K16" s="73">
+        <v>22</v>
+      </c>
+      <c r="L16" s="61">
+        <v>25.5</v>
+      </c>
+      <c r="M16" s="61">
+        <v>29.1</v>
+      </c>
+      <c r="N16" s="61">
+        <v>32.6</v>
+      </c>
+      <c r="O16" s="61">
+        <v>36.1</v>
+      </c>
+      <c r="P16" s="61">
+        <v>40.1</v>
+      </c>
+      <c r="Q16" s="61">
+        <v>23.7</v>
+      </c>
+      <c r="R16" s="61">
+        <v>27.3</v>
+      </c>
+      <c r="S16" s="61">
+        <v>30.7</v>
+      </c>
+      <c r="T16" s="61">
+        <v>34.200000000000003</v>
+      </c>
+      <c r="U16" s="61">
+        <v>38.200000000000003</v>
+      </c>
+      <c r="V16" s="61"/>
+      <c r="W16" s="70"/>
+    </row>
+    <row r="17" spans="1:23" x14ac:dyDescent="0.45">
+      <c r="A17" s="68"/>
+      <c r="B17" s="68" t="s">
         <v>100</v>
       </c>
-      <c r="C17" t="s">
+      <c r="C17" s="69">
+        <v>45054.415335648147</v>
+      </c>
+      <c r="D17" s="69">
+        <v>45054.421180555553</v>
+      </c>
+      <c r="E17" s="64" t="s">
         <v>258</v>
       </c>
-      <c r="D17" s="57" t="s">
+      <c r="F17" s="70" t="s">
         <v>260</v>
       </c>
-      <c r="F17" s="14" t="s">
+      <c r="H17" s="71" t="s">
         <v>271</v>
       </c>
-      <c r="G17" t="s">
+      <c r="I17" s="70" t="s">
         <v>280</v>
       </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A18" s="14"/>
-      <c r="B18" s="14" t="s">
+      <c r="K17" s="73">
+        <v>21.6</v>
+      </c>
+      <c r="L17" s="61">
+        <v>25.7</v>
+      </c>
+      <c r="M17" s="61">
+        <v>29.3</v>
+      </c>
+      <c r="N17" s="61">
+        <v>33.1</v>
+      </c>
+      <c r="O17" s="61">
+        <v>36.6</v>
+      </c>
+      <c r="P17" s="61">
+        <v>41.3</v>
+      </c>
+      <c r="Q17" s="61">
+        <v>24.2</v>
+      </c>
+      <c r="R17" s="61">
+        <v>27.8</v>
+      </c>
+      <c r="S17" s="61">
+        <v>31.3</v>
+      </c>
+      <c r="T17" s="61">
+        <v>34.9</v>
+      </c>
+      <c r="U17" s="61">
+        <v>38.6</v>
+      </c>
+      <c r="V17" s="61"/>
+      <c r="W17" s="70"/>
+    </row>
+    <row r="18" spans="1:23" x14ac:dyDescent="0.45">
+      <c r="A18" s="68"/>
+      <c r="B18" s="68" t="s">
         <v>101</v>
       </c>
-      <c r="C18" t="s">
+      <c r="C18" s="69">
+        <v>45055.170219907413</v>
+      </c>
+      <c r="D18" s="69">
+        <v>45055.199849537043</v>
+      </c>
+      <c r="E18" s="64" t="s">
         <v>258</v>
       </c>
-      <c r="D18" s="57" t="s">
+      <c r="F18" s="70" t="s">
         <v>260</v>
       </c>
-      <c r="F18" s="14" t="s">
+      <c r="H18" s="71" t="s">
         <v>271</v>
       </c>
-      <c r="G18" t="s">
+      <c r="I18" s="70" t="s">
         <v>280</v>
       </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A19" s="14"/>
-      <c r="B19" s="14" t="s">
+      <c r="K18" s="73">
+        <v>21.7</v>
+      </c>
+      <c r="L18" s="61">
+        <v>25.1</v>
+      </c>
+      <c r="M18" s="61">
+        <v>29</v>
+      </c>
+      <c r="N18" s="61">
+        <v>32.299999999999997</v>
+      </c>
+      <c r="O18" s="61"/>
+      <c r="P18" s="61"/>
+      <c r="Q18" s="61">
+        <v>23.6</v>
+      </c>
+      <c r="R18" s="61">
+        <v>27</v>
+      </c>
+      <c r="S18" s="61">
+        <v>31</v>
+      </c>
+      <c r="T18" s="61"/>
+      <c r="U18" s="61"/>
+      <c r="V18" s="61"/>
+      <c r="W18" s="70"/>
+    </row>
+    <row r="19" spans="1:23" x14ac:dyDescent="0.45">
+      <c r="A19" s="68"/>
+      <c r="B19" s="68" t="s">
         <v>102</v>
       </c>
-      <c r="C19" t="s">
+      <c r="C19" s="69">
+        <v>45055.351006944453</v>
+      </c>
+      <c r="D19" s="69">
+        <v>45055.355405092589</v>
+      </c>
+      <c r="E19" s="64" t="s">
         <v>258</v>
       </c>
-      <c r="D19" s="57" t="s">
+      <c r="F19" s="70" t="s">
         <v>260</v>
       </c>
-      <c r="F19" s="14" t="s">
+      <c r="H19" s="71" t="s">
         <v>271</v>
       </c>
-      <c r="G19" t="s">
+      <c r="I19" s="70" t="s">
         <v>280</v>
       </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A20" s="24"/>
-      <c r="B20" s="24" t="s">
+      <c r="K19" s="73">
+        <v>21.7</v>
+      </c>
+      <c r="L19" s="61">
+        <v>25.5</v>
+      </c>
+      <c r="M19" s="61">
+        <v>29.1</v>
+      </c>
+      <c r="N19" s="61">
+        <v>32.700000000000003</v>
+      </c>
+      <c r="O19" s="61"/>
+      <c r="P19" s="61"/>
+      <c r="Q19" s="61">
+        <v>23.4</v>
+      </c>
+      <c r="R19" s="61">
+        <v>27.3</v>
+      </c>
+      <c r="S19" s="61">
+        <v>31</v>
+      </c>
+      <c r="T19" s="61"/>
+      <c r="U19" s="61"/>
+      <c r="V19" s="61"/>
+      <c r="W19" s="70"/>
+    </row>
+    <row r="20" spans="1:23" x14ac:dyDescent="0.45">
+      <c r="A20" s="74"/>
+      <c r="B20" s="74" t="s">
         <v>269</v>
       </c>
-      <c r="C20" s="63" t="s">
+      <c r="C20" s="75">
+        <v>45055.378020833326</v>
+      </c>
+      <c r="D20" s="75">
+        <v>45055.399027777778</v>
+      </c>
+      <c r="E20" s="85" t="s">
         <v>258</v>
       </c>
-      <c r="D20" s="58" t="s">
+      <c r="F20" s="76" t="s">
         <v>260</v>
       </c>
-      <c r="F20" s="14" t="s">
+      <c r="H20" s="71" t="s">
         <v>271</v>
       </c>
-      <c r="G20" t="s">
+      <c r="I20" s="70" t="s">
         <v>280</v>
       </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A21" s="14" t="s">
+      <c r="K20" s="121">
+        <v>21.4</v>
+      </c>
+      <c r="L20" s="85">
+        <v>24.9</v>
+      </c>
+      <c r="M20" s="85">
+        <v>29</v>
+      </c>
+      <c r="N20" s="85">
+        <v>32.6</v>
+      </c>
+      <c r="O20" s="85">
+        <v>35.9</v>
+      </c>
+      <c r="P20" s="85">
+        <v>40.4</v>
+      </c>
+      <c r="Q20" s="85">
+        <v>23.1</v>
+      </c>
+      <c r="R20" s="85">
+        <v>27</v>
+      </c>
+      <c r="S20" s="85">
+        <v>30.8</v>
+      </c>
+      <c r="T20" s="85">
+        <v>34.4</v>
+      </c>
+      <c r="U20" s="85">
+        <v>37.6</v>
+      </c>
+      <c r="V20" s="85"/>
+      <c r="W20" s="76"/>
+    </row>
+    <row r="21" spans="1:23" x14ac:dyDescent="0.45">
+      <c r="A21" s="68" t="s">
         <v>30</v>
       </c>
-      <c r="B21" s="14" t="s">
+      <c r="B21" s="68" t="s">
         <v>106</v>
       </c>
-      <c r="C21" t="s">
+      <c r="C21" s="69">
+        <v>45119.225254629629</v>
+      </c>
+      <c r="D21" s="69">
+        <v>45119.260034722218</v>
+      </c>
+      <c r="E21" s="64" t="s">
         <v>258</v>
       </c>
-      <c r="D21" s="57" t="s">
+      <c r="F21" s="70" t="s">
         <v>260</v>
       </c>
-      <c r="F21" s="14" t="s">
+      <c r="H21" s="71" t="s">
         <v>271</v>
       </c>
-      <c r="G21" t="s">
+      <c r="I21" s="70" t="s">
         <v>280</v>
       </c>
-    </row>
-    <row r="22" spans="1:7" s="68" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="A22" s="11" t="s">
+      <c r="K21" s="122"/>
+      <c r="L21" s="79"/>
+      <c r="M21" s="79"/>
+      <c r="N21" s="79"/>
+      <c r="O21" s="79"/>
+      <c r="P21" s="79"/>
+      <c r="Q21" s="79"/>
+      <c r="R21" s="79"/>
+      <c r="S21" s="79"/>
+      <c r="T21" s="79"/>
+      <c r="U21" s="79"/>
+      <c r="V21" s="79"/>
+      <c r="W21" s="80"/>
+    </row>
+    <row r="22" spans="1:23" s="82" customFormat="1" x14ac:dyDescent="0.45">
+      <c r="A22" s="77" t="s">
         <v>31</v>
       </c>
-      <c r="B22" s="11" t="s">
+      <c r="B22" s="77" t="s">
         <v>108</v>
       </c>
-      <c r="C22" s="62" t="s">
+      <c r="C22" s="78">
+        <v>45122.301076388889</v>
+      </c>
+      <c r="D22" s="78">
+        <v>45122.310162037036</v>
+      </c>
+      <c r="E22" s="79" t="s">
         <v>257</v>
       </c>
-      <c r="D22" s="61" t="s">
+      <c r="F22" s="80" t="s">
         <v>260</v>
       </c>
-      <c r="E22"/>
-      <c r="F22" s="14" t="s">
+      <c r="G22" s="64"/>
+      <c r="H22" s="71" t="s">
         <v>271</v>
       </c>
-      <c r="G22" t="s">
+      <c r="I22" s="70" t="s">
         <v>280</v>
       </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A23" s="51" t="s">
+      <c r="K22" s="123"/>
+      <c r="L22" s="100"/>
+      <c r="M22" s="100"/>
+      <c r="N22" s="100"/>
+      <c r="O22" s="100"/>
+      <c r="P22" s="100"/>
+      <c r="Q22" s="100"/>
+      <c r="R22" s="100"/>
+      <c r="S22" s="100"/>
+      <c r="T22" s="100"/>
+      <c r="U22" s="100"/>
+      <c r="V22" s="100"/>
+      <c r="W22" s="101"/>
+    </row>
+    <row r="23" spans="1:23" x14ac:dyDescent="0.45">
+      <c r="A23" s="86" t="s">
         <v>32</v>
       </c>
-      <c r="B23" s="26" t="s">
+      <c r="B23" s="90" t="s">
         <v>109</v>
       </c>
-      <c r="C23" s="66" t="s">
+      <c r="C23" s="99"/>
+      <c r="D23" s="99"/>
+      <c r="E23" s="100" t="s">
         <v>257</v>
       </c>
-      <c r="D23" s="67" t="s">
+      <c r="F23" s="101" t="s">
         <v>261</v>
       </c>
-      <c r="E23" s="68" t="s">
+      <c r="G23" s="82" t="s">
         <v>262</v>
       </c>
-      <c r="F23" s="26" t="s">
+      <c r="H23" s="92" t="s">
         <v>271</v>
       </c>
-    </row>
-    <row r="24" spans="1:7" s="68" customFormat="1" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A24" s="59" t="s">
+      <c r="I23" s="70"/>
+      <c r="K23" s="122"/>
+      <c r="L23" s="79"/>
+      <c r="M23" s="79"/>
+      <c r="N23" s="79"/>
+      <c r="O23" s="79"/>
+      <c r="P23" s="79"/>
+      <c r="Q23" s="79"/>
+      <c r="R23" s="79"/>
+      <c r="S23" s="79"/>
+      <c r="T23" s="79"/>
+      <c r="U23" s="79"/>
+      <c r="V23" s="79"/>
+      <c r="W23" s="80"/>
+    </row>
+    <row r="24" spans="1:23" s="82" customFormat="1" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A24" s="102" t="s">
         <v>33</v>
       </c>
-      <c r="B24" s="59" t="s">
+      <c r="B24" s="102" t="s">
         <v>110</v>
       </c>
-      <c r="C24" s="60" t="s">
+      <c r="C24" s="103">
+        <v>45143.215335648143</v>
+      </c>
+      <c r="D24" s="103">
+        <v>45143.242708333331</v>
+      </c>
+      <c r="E24" s="63" t="s">
         <v>258</v>
       </c>
-      <c r="D24" s="65" t="s">
+      <c r="F24" s="104" t="s">
         <v>260</v>
       </c>
-      <c r="E24"/>
-      <c r="F24" s="14" t="s">
+      <c r="G24" s="64"/>
+      <c r="H24" s="105" t="s">
         <v>272</v>
       </c>
-      <c r="G24" t="s">
+      <c r="I24" s="106" t="s">
         <v>280</v>
       </c>
-    </row>
-    <row r="25" spans="1:7" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="A25" s="14" t="s">
+      <c r="K24" s="126"/>
+      <c r="L24" s="127"/>
+      <c r="M24" s="127"/>
+      <c r="N24" s="127"/>
+      <c r="O24" s="127"/>
+      <c r="P24" s="127"/>
+      <c r="Q24" s="127"/>
+      <c r="R24" s="127"/>
+      <c r="S24" s="127"/>
+      <c r="T24" s="127"/>
+      <c r="U24" s="127"/>
+      <c r="V24" s="127"/>
+      <c r="W24" s="128"/>
+    </row>
+    <row r="25" spans="1:23" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
+      <c r="A25" s="68" t="s">
         <v>40</v>
       </c>
-      <c r="B25" s="14" t="s">
+      <c r="B25" s="68" t="s">
         <v>140</v>
       </c>
-      <c r="C25" t="s">
+      <c r="C25" s="69">
+        <v>43358.436255787034</v>
+      </c>
+      <c r="D25" s="68"/>
+      <c r="E25" s="64" t="s">
         <v>257</v>
       </c>
-      <c r="D25" s="57" t="s">
+      <c r="F25" s="70" t="s">
         <v>260</v>
       </c>
-      <c r="E25" s="69"/>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A26" s="14"/>
-      <c r="B26" s="14" t="s">
+      <c r="G25" s="89" t="s">
+        <v>296</v>
+      </c>
+      <c r="K25" s="73"/>
+      <c r="L25" s="61"/>
+      <c r="M25" s="61"/>
+      <c r="N25" s="61"/>
+      <c r="O25" s="61"/>
+      <c r="P25" s="61"/>
+      <c r="Q25" s="61"/>
+      <c r="R25" s="61"/>
+      <c r="S25" s="61"/>
+      <c r="T25" s="61"/>
+      <c r="U25" s="61"/>
+      <c r="V25" s="61"/>
+      <c r="W25" s="70"/>
+    </row>
+    <row r="26" spans="1:23" x14ac:dyDescent="0.45">
+      <c r="A26" s="68"/>
+      <c r="B26" s="68" t="s">
         <v>141</v>
       </c>
-      <c r="C26" t="s">
+      <c r="C26" s="69">
+        <v>43358.450086805547</v>
+      </c>
+      <c r="D26" s="68"/>
+      <c r="E26" s="64" t="s">
         <v>258</v>
       </c>
-      <c r="D26" s="57" t="s">
+      <c r="F26" s="70" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A27" s="14"/>
-      <c r="B27" s="14" t="s">
+      <c r="K26" s="73"/>
+      <c r="L26" s="61"/>
+      <c r="M26" s="61"/>
+      <c r="N26" s="61"/>
+      <c r="O26" s="61"/>
+      <c r="P26" s="61"/>
+      <c r="Q26" s="61"/>
+      <c r="R26" s="61"/>
+      <c r="S26" s="61"/>
+      <c r="T26" s="61"/>
+      <c r="U26" s="61"/>
+      <c r="V26" s="61"/>
+      <c r="W26" s="70"/>
+    </row>
+    <row r="27" spans="1:23" x14ac:dyDescent="0.45">
+      <c r="A27" s="68"/>
+      <c r="B27" s="68" t="s">
         <v>142</v>
       </c>
-      <c r="C27" t="s">
+      <c r="C27" s="69">
+        <v>43358.464033564807</v>
+      </c>
+      <c r="D27" s="68"/>
+      <c r="E27" s="64" t="s">
         <v>258</v>
       </c>
-      <c r="D27" s="57" t="s">
+      <c r="F27" s="70" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="28" spans="1:7" s="68" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="A28" s="29"/>
-      <c r="B28" s="29" t="s">
+      <c r="K27" s="73"/>
+      <c r="L27" s="61"/>
+      <c r="M27" s="61"/>
+      <c r="N27" s="61"/>
+      <c r="O27" s="61"/>
+      <c r="P27" s="61"/>
+      <c r="Q27" s="61"/>
+      <c r="R27" s="61"/>
+      <c r="S27" s="61"/>
+      <c r="T27" s="61"/>
+      <c r="U27" s="61"/>
+      <c r="V27" s="61"/>
+      <c r="W27" s="70"/>
+    </row>
+    <row r="28" spans="1:23" s="82" customFormat="1" x14ac:dyDescent="0.45">
+      <c r="A28" s="107"/>
+      <c r="B28" s="107" t="s">
         <v>143</v>
       </c>
-      <c r="C28" s="70" t="s">
+      <c r="C28" s="107"/>
+      <c r="D28" s="107"/>
+      <c r="E28" s="108" t="s">
         <v>258</v>
       </c>
-      <c r="D28" s="71" t="s">
+      <c r="F28" s="109" t="s">
         <v>260</v>
       </c>
-      <c r="E28" s="68" t="s">
+      <c r="G28" s="82" t="s">
         <v>262</v>
       </c>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A29" s="14" t="s">
+      <c r="K28" s="124"/>
+      <c r="L28" s="108"/>
+      <c r="M28" s="108"/>
+      <c r="N28" s="108"/>
+      <c r="O28" s="108"/>
+      <c r="P28" s="108"/>
+      <c r="Q28" s="108"/>
+      <c r="R28" s="108"/>
+      <c r="S28" s="108"/>
+      <c r="T28" s="108"/>
+      <c r="U28" s="108"/>
+      <c r="V28" s="108"/>
+      <c r="W28" s="109"/>
+    </row>
+    <row r="29" spans="1:23" x14ac:dyDescent="0.45">
+      <c r="A29" s="68" t="s">
         <v>41</v>
       </c>
-      <c r="B29" s="14" t="s">
+      <c r="B29" s="68" t="s">
         <v>144</v>
       </c>
-      <c r="C29" t="s">
+      <c r="C29" s="69">
+        <v>43338.193541666667</v>
+      </c>
+      <c r="D29" s="68"/>
+      <c r="E29" s="64" t="s">
         <v>257</v>
       </c>
-      <c r="D29" s="57" t="s">
+      <c r="F29" s="70" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A30" s="14"/>
-      <c r="B30" s="14" t="s">
+      <c r="G29" s="89" t="s">
+        <v>297</v>
+      </c>
+      <c r="K29" s="129"/>
+      <c r="L29" s="61"/>
+      <c r="M29" s="61"/>
+      <c r="N29" s="61"/>
+      <c r="O29" s="61"/>
+      <c r="P29" s="61"/>
+      <c r="Q29" s="61"/>
+      <c r="R29" s="61"/>
+      <c r="S29" s="61"/>
+      <c r="T29" s="61"/>
+      <c r="U29" s="61"/>
+      <c r="V29" s="61"/>
+      <c r="W29" s="70"/>
+    </row>
+    <row r="30" spans="1:23" x14ac:dyDescent="0.45">
+      <c r="A30" s="68"/>
+      <c r="B30" s="68" t="s">
         <v>145</v>
       </c>
-      <c r="C30" t="s">
+      <c r="C30" s="69">
+        <v>43338.207309027777</v>
+      </c>
+      <c r="D30" s="68"/>
+      <c r="E30" s="64" t="s">
         <v>258</v>
       </c>
-      <c r="D30" s="57" t="s">
+      <c r="F30" s="70" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A31" s="26"/>
-      <c r="B31" s="14" t="s">
+      <c r="J30" s="70"/>
+      <c r="K30" s="73">
+        <v>20.8</v>
+      </c>
+      <c r="L30" s="61">
+        <v>24.1</v>
+      </c>
+      <c r="M30" s="61">
+        <v>28</v>
+      </c>
+      <c r="N30" s="61">
+        <v>30.9</v>
+      </c>
+      <c r="O30" s="61"/>
+      <c r="P30" s="61"/>
+      <c r="Q30" s="61">
+        <v>22.3</v>
+      </c>
+      <c r="R30" s="61">
+        <v>25.7</v>
+      </c>
+      <c r="S30" s="61">
+        <v>29.3</v>
+      </c>
+      <c r="T30" s="61"/>
+      <c r="U30" s="61"/>
+      <c r="V30" s="61" t="s">
+        <v>272</v>
+      </c>
+      <c r="W30" s="70" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="31" spans="1:23" x14ac:dyDescent="0.45">
+      <c r="A31" s="90"/>
+      <c r="B31" s="68" t="s">
         <v>147</v>
       </c>
-      <c r="C31" t="s">
+      <c r="C31" s="69">
+        <v>43339.277042824076</v>
+      </c>
+      <c r="D31" s="68"/>
+      <c r="E31" s="64" t="s">
         <v>258</v>
       </c>
-      <c r="D31" s="57" t="s">
+      <c r="F31" s="70" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A32" s="14"/>
-      <c r="B32" s="14" t="s">
+      <c r="K31" s="73">
+        <v>21.2</v>
+      </c>
+      <c r="L31" s="61">
+        <v>24.4</v>
+      </c>
+      <c r="M31" s="61">
+        <v>28.4</v>
+      </c>
+      <c r="N31" s="61">
+        <v>31.8</v>
+      </c>
+      <c r="O31" s="61"/>
+      <c r="P31" s="61"/>
+      <c r="Q31" s="61">
+        <v>22.6</v>
+      </c>
+      <c r="R31" s="61">
+        <v>26.2</v>
+      </c>
+      <c r="S31" s="61">
+        <v>29.6</v>
+      </c>
+      <c r="T31" s="61"/>
+      <c r="U31" s="61"/>
+      <c r="V31" s="61" t="s">
+        <v>272</v>
+      </c>
+      <c r="W31" s="70" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="32" spans="1:23" x14ac:dyDescent="0.45">
+      <c r="A32" s="68"/>
+      <c r="B32" s="68" t="s">
         <v>148</v>
       </c>
-      <c r="C32" t="s">
+      <c r="C32" s="69">
+        <v>43339.290700231482</v>
+      </c>
+      <c r="D32" s="68"/>
+      <c r="E32" s="64" t="s">
         <v>258</v>
       </c>
-      <c r="D32" s="57" t="s">
+      <c r="F32" s="70" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A33" s="14"/>
-      <c r="B33" s="14" t="s">
+      <c r="K32" s="73">
+        <v>20.9</v>
+      </c>
+      <c r="L32" s="61">
+        <v>24.4</v>
+      </c>
+      <c r="M32" s="61">
+        <v>27.9</v>
+      </c>
+      <c r="N32" s="61">
+        <v>31.6</v>
+      </c>
+      <c r="O32" s="61"/>
+      <c r="P32" s="61"/>
+      <c r="Q32" s="61">
+        <v>22.3</v>
+      </c>
+      <c r="R32" s="61">
+        <v>26</v>
+      </c>
+      <c r="S32" s="61">
+        <v>28.8</v>
+      </c>
+      <c r="T32" s="61"/>
+      <c r="U32" s="61"/>
+      <c r="V32" s="61" t="s">
+        <v>272</v>
+      </c>
+      <c r="W32" s="70" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="33" spans="1:23" x14ac:dyDescent="0.45">
+      <c r="A33" s="68"/>
+      <c r="B33" s="68" t="s">
         <v>150</v>
       </c>
-      <c r="C33" t="s">
+      <c r="C33" s="69">
+        <v>43339.734913194443</v>
+      </c>
+      <c r="D33" s="68"/>
+      <c r="E33" s="64" t="s">
         <v>258</v>
       </c>
-      <c r="D33" s="57" t="s">
+      <c r="F33" s="70" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A34" s="26"/>
-      <c r="B34" s="14" t="s">
+      <c r="K33" s="73">
+        <v>20.2</v>
+      </c>
+      <c r="L33" s="61">
+        <v>23.6</v>
+      </c>
+      <c r="M33" s="61">
+        <v>27.4</v>
+      </c>
+      <c r="N33" s="61">
+        <v>31.3</v>
+      </c>
+      <c r="O33" s="61"/>
+      <c r="P33" s="61"/>
+      <c r="Q33" s="61">
+        <v>21.9</v>
+      </c>
+      <c r="R33" s="61">
+        <v>25.5</v>
+      </c>
+      <c r="S33" s="61">
+        <v>28.8</v>
+      </c>
+      <c r="T33" s="61"/>
+      <c r="U33" s="61"/>
+      <c r="V33" s="61" t="s">
+        <v>272</v>
+      </c>
+      <c r="W33" s="70" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="34" spans="1:23" x14ac:dyDescent="0.45">
+      <c r="A34" s="90"/>
+      <c r="B34" s="68" t="s">
         <v>151</v>
       </c>
-      <c r="C34" t="s">
+      <c r="C34" s="69">
+        <v>43344.179531250003</v>
+      </c>
+      <c r="D34" s="68"/>
+      <c r="E34" s="64" t="s">
         <v>258</v>
       </c>
-      <c r="D34" s="57" t="s">
+      <c r="F34" s="70" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A35" s="14"/>
-      <c r="B35" s="14" t="s">
+      <c r="K34" s="73">
+        <v>20.8</v>
+      </c>
+      <c r="L34" s="61">
+        <v>24.3</v>
+      </c>
+      <c r="M34" s="61">
+        <v>28.1</v>
+      </c>
+      <c r="N34" s="61">
+        <v>31.5</v>
+      </c>
+      <c r="O34" s="61"/>
+      <c r="P34" s="61"/>
+      <c r="Q34" s="61">
+        <v>22.9</v>
+      </c>
+      <c r="R34" s="61">
+        <v>26.7</v>
+      </c>
+      <c r="S34" s="61">
+        <v>30.2</v>
+      </c>
+      <c r="T34" s="61"/>
+      <c r="U34" s="61"/>
+      <c r="V34" s="61" t="s">
+        <v>272</v>
+      </c>
+      <c r="W34" s="70" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="35" spans="1:23" x14ac:dyDescent="0.45">
+      <c r="A35" s="68"/>
+      <c r="B35" s="68" t="s">
         <v>152</v>
       </c>
-      <c r="C35" t="s">
+      <c r="C35" s="69">
+        <v>43344.193420138887</v>
+      </c>
+      <c r="D35" s="68"/>
+      <c r="E35" s="64" t="s">
         <v>258</v>
       </c>
-      <c r="D35" s="57" t="s">
+      <c r="F35" s="70" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A36" s="26"/>
-      <c r="B36" s="14" t="s">
+      <c r="K35" s="73">
+        <v>21</v>
+      </c>
+      <c r="L35" s="61">
+        <v>24.1</v>
+      </c>
+      <c r="M35" s="61">
+        <v>27.8</v>
+      </c>
+      <c r="N35" s="61">
+        <v>32.200000000000003</v>
+      </c>
+      <c r="O35" s="61"/>
+      <c r="P35" s="61"/>
+      <c r="Q35" s="61">
+        <v>22.7</v>
+      </c>
+      <c r="R35" s="61">
+        <v>26.4</v>
+      </c>
+      <c r="S35" s="61">
+        <v>30</v>
+      </c>
+      <c r="T35" s="61"/>
+      <c r="U35" s="61"/>
+      <c r="V35" s="61" t="s">
+        <v>272</v>
+      </c>
+      <c r="W35" s="70" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="36" spans="1:23" x14ac:dyDescent="0.45">
+      <c r="A36" s="90"/>
+      <c r="B36" s="68" t="s">
         <v>153</v>
       </c>
-      <c r="C36" t="s">
+      <c r="C36" s="69">
+        <v>43345.248917824079</v>
+      </c>
+      <c r="D36" s="68"/>
+      <c r="E36" s="64" t="s">
         <v>258</v>
       </c>
-      <c r="D36" s="57" t="s">
+      <c r="F36" s="70" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A37" s="14"/>
-      <c r="B37" s="14" t="s">
+      <c r="K36" s="73">
+        <v>20.8</v>
+      </c>
+      <c r="L36" s="61">
+        <v>24.1</v>
+      </c>
+      <c r="M36" s="61"/>
+      <c r="N36" s="61"/>
+      <c r="O36" s="61"/>
+      <c r="P36" s="61"/>
+      <c r="Q36" s="61">
+        <v>22.3</v>
+      </c>
+      <c r="R36" s="61">
+        <v>26.2</v>
+      </c>
+      <c r="S36" s="61"/>
+      <c r="T36" s="61"/>
+      <c r="U36" s="61"/>
+      <c r="V36" s="61"/>
+      <c r="W36" s="70"/>
+    </row>
+    <row r="37" spans="1:23" x14ac:dyDescent="0.45">
+      <c r="A37" s="68"/>
+      <c r="B37" s="68" t="s">
         <v>154</v>
       </c>
-      <c r="C37" t="s">
+      <c r="C37" s="69">
+        <v>43345.262748842593</v>
+      </c>
+      <c r="D37" s="68"/>
+      <c r="E37" s="64" t="s">
         <v>257</v>
       </c>
-      <c r="D37" s="57" t="s">
+      <c r="F37" s="70" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A38" s="14"/>
-      <c r="B38" s="14" t="s">
+      <c r="K37" s="73">
+        <v>20.2</v>
+      </c>
+      <c r="L37" s="61">
+        <v>23.6</v>
+      </c>
+      <c r="M37" s="61">
+        <v>28.3</v>
+      </c>
+      <c r="N37" s="61">
+        <v>31.6</v>
+      </c>
+      <c r="O37" s="61"/>
+      <c r="P37" s="61"/>
+      <c r="Q37" s="61">
+        <v>22.2</v>
+      </c>
+      <c r="R37" s="61">
+        <v>25.7</v>
+      </c>
+      <c r="S37" s="61">
+        <v>29.5</v>
+      </c>
+      <c r="T37" s="61"/>
+      <c r="U37" s="61"/>
+      <c r="V37" s="61"/>
+      <c r="W37" s="70"/>
+    </row>
+    <row r="38" spans="1:23" x14ac:dyDescent="0.45">
+      <c r="A38" s="68"/>
+      <c r="B38" s="68" t="s">
         <v>156</v>
       </c>
-      <c r="C38" t="s">
+      <c r="C38" s="69">
+        <v>43345.457366898147</v>
+      </c>
+      <c r="D38" s="68"/>
+      <c r="E38" s="64" t="s">
         <v>258</v>
       </c>
-      <c r="D38" s="57" t="s">
+      <c r="F38" s="70" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="39" spans="1:5" s="68" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="A39" s="26"/>
-      <c r="B39" s="26" t="s">
+      <c r="K38" s="73">
+        <v>20.8</v>
+      </c>
+      <c r="L38" s="61">
+        <v>24.3</v>
+      </c>
+      <c r="M38" s="61">
+        <v>28.3</v>
+      </c>
+      <c r="N38" s="61">
+        <v>31.7</v>
+      </c>
+      <c r="O38" s="61"/>
+      <c r="P38" s="61"/>
+      <c r="Q38" s="61">
+        <v>22.8</v>
+      </c>
+      <c r="R38" s="61">
+        <v>26.2</v>
+      </c>
+      <c r="S38" s="61">
+        <v>30.1</v>
+      </c>
+      <c r="T38" s="61"/>
+      <c r="U38" s="61"/>
+      <c r="V38" s="61"/>
+      <c r="W38" s="70"/>
+    </row>
+    <row r="39" spans="1:23" s="82" customFormat="1" x14ac:dyDescent="0.45">
+      <c r="A39" s="90"/>
+      <c r="B39" s="90" t="s">
         <v>164</v>
       </c>
-      <c r="C39" s="68" t="s">
+      <c r="C39" s="90"/>
+      <c r="D39" s="90"/>
+      <c r="E39" s="82" t="s">
         <v>257</v>
       </c>
-      <c r="D39" s="72" t="s">
+      <c r="F39" s="84" t="s">
         <v>261</v>
       </c>
-      <c r="E39" s="68" t="s">
+      <c r="G39" s="82" t="s">
         <v>262</v>
       </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A40" s="26"/>
-      <c r="B40" s="14" t="s">
+      <c r="K39" s="83"/>
+      <c r="L39" s="62"/>
+      <c r="M39" s="62"/>
+      <c r="N39" s="62"/>
+      <c r="O39" s="62"/>
+      <c r="P39" s="62"/>
+      <c r="Q39" s="62"/>
+      <c r="R39" s="62"/>
+      <c r="S39" s="62"/>
+      <c r="T39" s="62"/>
+      <c r="U39" s="62"/>
+      <c r="V39" s="62"/>
+      <c r="W39" s="84"/>
+    </row>
+    <row r="40" spans="1:23" x14ac:dyDescent="0.45">
+      <c r="A40" s="90"/>
+      <c r="B40" s="68" t="s">
         <v>166</v>
       </c>
-      <c r="C40" t="s">
+      <c r="C40" s="69">
+        <v>43357.471313657406</v>
+      </c>
+      <c r="D40" s="68"/>
+      <c r="E40" s="64" t="s">
         <v>258</v>
       </c>
-      <c r="D40" s="57" t="s">
+      <c r="F40" s="70" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A41" s="14"/>
-      <c r="B41" s="14" t="s">
+      <c r="K40" s="73">
+        <v>20.399999999999999</v>
+      </c>
+      <c r="L40" s="61">
+        <v>24.1</v>
+      </c>
+      <c r="M40" s="61">
+        <v>27.2</v>
+      </c>
+      <c r="N40" s="61">
+        <v>30.7</v>
+      </c>
+      <c r="O40" s="61"/>
+      <c r="P40" s="61"/>
+      <c r="Q40" s="61">
+        <v>22.6</v>
+      </c>
+      <c r="R40" s="61">
+        <v>25.7</v>
+      </c>
+      <c r="S40" s="61">
+        <v>28.7</v>
+      </c>
+      <c r="T40" s="61"/>
+      <c r="U40" s="61"/>
+      <c r="V40" s="61"/>
+      <c r="W40" s="70"/>
+    </row>
+    <row r="41" spans="1:23" x14ac:dyDescent="0.45">
+      <c r="A41" s="68"/>
+      <c r="B41" s="68" t="s">
         <v>167</v>
       </c>
-      <c r="C41" t="s">
+      <c r="C41" s="69">
+        <v>43358.318188657402</v>
+      </c>
+      <c r="D41" s="68"/>
+      <c r="E41" s="64" t="s">
         <v>258</v>
       </c>
-      <c r="D41" s="57" t="s">
+      <c r="F41" s="70" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A42" s="14"/>
-      <c r="B42" s="14" t="s">
+      <c r="K41" s="73">
+        <v>20.8</v>
+      </c>
+      <c r="L41" s="61">
+        <v>23.8</v>
+      </c>
+      <c r="M41" s="61">
+        <v>27.6</v>
+      </c>
+      <c r="N41" s="61">
+        <v>31.5</v>
+      </c>
+      <c r="O41" s="61"/>
+      <c r="P41" s="61"/>
+      <c r="Q41" s="61">
+        <v>22.3</v>
+      </c>
+      <c r="R41" s="61">
+        <v>25.7</v>
+      </c>
+      <c r="S41" s="61">
+        <v>29.2</v>
+      </c>
+      <c r="T41" s="61"/>
+      <c r="U41" s="61"/>
+      <c r="V41" s="61"/>
+      <c r="W41" s="70"/>
+    </row>
+    <row r="42" spans="1:23" x14ac:dyDescent="0.45">
+      <c r="A42" s="68"/>
+      <c r="B42" s="68" t="s">
         <v>168</v>
       </c>
-      <c r="C42" t="s">
+      <c r="C42" s="69">
+        <v>43359.318651620371</v>
+      </c>
+      <c r="D42" s="68"/>
+      <c r="E42" s="64" t="s">
         <v>257</v>
       </c>
-      <c r="D42" s="57" t="s">
+      <c r="F42" s="70" t="s">
         <v>260</v>
       </c>
-      <c r="E42" t="s">
-        <v>281</v>
-      </c>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A43" s="26"/>
-      <c r="B43" s="14" t="s">
+      <c r="K42" s="73"/>
+      <c r="L42" s="61"/>
+      <c r="M42" s="61"/>
+      <c r="N42" s="61"/>
+      <c r="O42" s="61"/>
+      <c r="P42" s="61"/>
+      <c r="Q42" s="61"/>
+      <c r="R42" s="61"/>
+      <c r="S42" s="61"/>
+      <c r="T42" s="61"/>
+      <c r="U42" s="61"/>
+      <c r="V42" s="61"/>
+      <c r="W42" s="70"/>
+    </row>
+    <row r="43" spans="1:23" x14ac:dyDescent="0.45">
+      <c r="A43" s="90"/>
+      <c r="B43" s="68" t="s">
         <v>170</v>
       </c>
-      <c r="C43" t="s">
+      <c r="C43" s="69">
+        <v>43367.123802083333</v>
+      </c>
+      <c r="D43" s="68"/>
+      <c r="E43" s="64" t="s">
         <v>258</v>
       </c>
-      <c r="D43" s="57" t="s">
+      <c r="F43" s="70" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A44" s="26"/>
-      <c r="B44" s="14" t="s">
+      <c r="K43" s="73"/>
+      <c r="L43" s="61"/>
+      <c r="M43" s="61"/>
+      <c r="N43" s="61"/>
+      <c r="O43" s="61"/>
+      <c r="P43" s="61"/>
+      <c r="Q43" s="61"/>
+      <c r="R43" s="61"/>
+      <c r="S43" s="61"/>
+      <c r="T43" s="61"/>
+      <c r="U43" s="61"/>
+      <c r="V43" s="61"/>
+      <c r="W43" s="70"/>
+    </row>
+    <row r="44" spans="1:23" x14ac:dyDescent="0.45">
+      <c r="A44" s="90"/>
+      <c r="B44" s="68" t="s">
         <v>171</v>
       </c>
-      <c r="C44" t="s">
+      <c r="C44" s="69">
+        <v>43367.138211805563</v>
+      </c>
+      <c r="D44" s="68"/>
+      <c r="E44" s="64" t="s">
         <v>258</v>
       </c>
-      <c r="D44" s="57" t="s">
+      <c r="F44" s="70" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A45" s="26"/>
-      <c r="B45" s="14" t="s">
+      <c r="K44" s="73">
+        <v>20.8</v>
+      </c>
+      <c r="L44" s="61">
+        <v>24.5</v>
+      </c>
+      <c r="M44" s="61">
+        <v>28.3</v>
+      </c>
+      <c r="N44" s="61">
+        <v>31.9</v>
+      </c>
+      <c r="O44" s="61"/>
+      <c r="P44" s="61"/>
+      <c r="Q44" s="61">
+        <v>22.6</v>
+      </c>
+      <c r="R44" s="61">
+        <v>25.7</v>
+      </c>
+      <c r="S44" s="61">
+        <v>30</v>
+      </c>
+      <c r="T44" s="61"/>
+      <c r="U44" s="61"/>
+      <c r="V44" s="61"/>
+      <c r="W44" s="70"/>
+    </row>
+    <row r="45" spans="1:23" x14ac:dyDescent="0.45">
+      <c r="A45" s="90"/>
+      <c r="B45" s="68" t="s">
         <v>173</v>
       </c>
-      <c r="C45" t="s">
+      <c r="C45" s="69">
+        <v>43368.346197916668</v>
+      </c>
+      <c r="D45" s="68"/>
+      <c r="E45" s="64" t="s">
         <v>258</v>
       </c>
-      <c r="D45" s="57" t="s">
+      <c r="F45" s="70" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A46" s="26"/>
-      <c r="B46" s="14" t="s">
+      <c r="K45" s="73">
+        <v>21</v>
+      </c>
+      <c r="L45" s="61">
+        <v>24.2</v>
+      </c>
+      <c r="M45" s="61">
+        <v>27.9</v>
+      </c>
+      <c r="N45" s="61">
+        <v>31</v>
+      </c>
+      <c r="O45" s="61"/>
+      <c r="P45" s="61"/>
+      <c r="Q45" s="61">
+        <v>22.7</v>
+      </c>
+      <c r="R45" s="61">
+        <v>26.1</v>
+      </c>
+      <c r="S45" s="61">
+        <v>29.2</v>
+      </c>
+      <c r="T45" s="61"/>
+      <c r="U45" s="61"/>
+      <c r="V45" s="61"/>
+      <c r="W45" s="70"/>
+    </row>
+    <row r="46" spans="1:23" x14ac:dyDescent="0.45">
+      <c r="A46" s="90"/>
+      <c r="B46" s="68" t="s">
         <v>174</v>
       </c>
-      <c r="C46" t="s">
+      <c r="C46" s="69">
+        <v>43368.359971064812</v>
+      </c>
+      <c r="D46" s="68"/>
+      <c r="E46" s="64" t="s">
         <v>258</v>
       </c>
-      <c r="D46" s="57" t="s">
+      <c r="F46" s="70" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="47" spans="1:5" s="68" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="A47" s="26"/>
-      <c r="B47" s="26" t="s">
+      <c r="K46" s="73">
+        <v>21.2</v>
+      </c>
+      <c r="L46" s="61">
+        <v>24.5</v>
+      </c>
+      <c r="M46" s="61">
+        <v>28.2</v>
+      </c>
+      <c r="N46" s="61">
+        <v>30.9</v>
+      </c>
+      <c r="O46" s="61"/>
+      <c r="P46" s="61"/>
+      <c r="Q46" s="61">
+        <v>22.9</v>
+      </c>
+      <c r="R46" s="61">
+        <v>26.1</v>
+      </c>
+      <c r="S46" s="61">
+        <v>29.6</v>
+      </c>
+      <c r="T46" s="61"/>
+      <c r="U46" s="61"/>
+      <c r="V46" s="61"/>
+      <c r="W46" s="70"/>
+    </row>
+    <row r="47" spans="1:23" s="82" customFormat="1" x14ac:dyDescent="0.45">
+      <c r="A47" s="90"/>
+      <c r="B47" s="90" t="s">
         <v>175</v>
       </c>
-      <c r="C47" s="68" t="s">
+      <c r="C47" s="90"/>
+      <c r="D47" s="90"/>
+      <c r="E47" s="82" t="s">
         <v>257</v>
       </c>
-      <c r="D47" s="72" t="s">
+      <c r="F47" s="84" t="s">
         <v>261</v>
       </c>
-      <c r="E47" s="68" t="s">
+      <c r="G47" s="82" t="s">
         <v>262</v>
       </c>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A48" s="26"/>
-      <c r="B48" s="14" t="s">
+      <c r="K47" s="83"/>
+      <c r="L47" s="62"/>
+      <c r="M47" s="62"/>
+      <c r="N47" s="62"/>
+      <c r="O47" s="62"/>
+      <c r="P47" s="62"/>
+      <c r="Q47" s="62"/>
+      <c r="R47" s="62"/>
+      <c r="S47" s="62"/>
+      <c r="T47" s="62"/>
+      <c r="U47" s="62"/>
+      <c r="V47" s="62"/>
+      <c r="W47" s="84"/>
+    </row>
+    <row r="48" spans="1:23" x14ac:dyDescent="0.45">
+      <c r="A48" s="90"/>
+      <c r="B48" s="68" t="s">
         <v>176</v>
       </c>
-      <c r="C48" t="s">
+      <c r="C48" s="69">
+        <v>43370.304704861112</v>
+      </c>
+      <c r="D48" s="68"/>
+      <c r="E48" s="64" t="s">
         <v>258</v>
       </c>
-      <c r="D48" s="57" t="s">
+      <c r="F48" s="70" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="49" spans="1:5" s="68" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="A49" s="26"/>
-      <c r="B49" s="26" t="s">
+      <c r="K48" s="73"/>
+      <c r="L48" s="61"/>
+      <c r="M48" s="61"/>
+      <c r="N48" s="61"/>
+      <c r="O48" s="61"/>
+      <c r="P48" s="61"/>
+      <c r="Q48" s="61"/>
+      <c r="R48" s="61"/>
+      <c r="S48" s="61"/>
+      <c r="T48" s="61"/>
+      <c r="U48" s="61"/>
+      <c r="V48" s="61"/>
+      <c r="W48" s="70"/>
+    </row>
+    <row r="49" spans="1:23" s="82" customFormat="1" x14ac:dyDescent="0.45">
+      <c r="A49" s="90"/>
+      <c r="B49" s="90" t="s">
         <v>180</v>
       </c>
-      <c r="C49" s="68" t="s">
+      <c r="C49" s="90"/>
+      <c r="D49" s="90"/>
+      <c r="E49" s="82" t="s">
         <v>257</v>
       </c>
-      <c r="D49" s="72" t="s">
+      <c r="F49" s="84" t="s">
         <v>261</v>
       </c>
-      <c r="E49" s="68" t="s">
+      <c r="G49" s="82" t="s">
         <v>262</v>
       </c>
-    </row>
-    <row r="50" spans="1:5" s="68" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="A50" s="29"/>
-      <c r="B50" s="29" t="s">
+      <c r="K49" s="83"/>
+      <c r="L49" s="62"/>
+      <c r="M49" s="62"/>
+      <c r="N49" s="62"/>
+      <c r="O49" s="62"/>
+      <c r="P49" s="62"/>
+      <c r="Q49" s="62"/>
+      <c r="R49" s="62"/>
+      <c r="S49" s="62"/>
+      <c r="T49" s="62"/>
+      <c r="U49" s="62"/>
+      <c r="V49" s="62"/>
+      <c r="W49" s="84"/>
+    </row>
+    <row r="50" spans="1:23" s="82" customFormat="1" x14ac:dyDescent="0.45">
+      <c r="A50" s="107"/>
+      <c r="B50" s="107" t="s">
         <v>181</v>
       </c>
-      <c r="C50" s="70" t="s">
+      <c r="C50" s="107"/>
+      <c r="D50" s="107"/>
+      <c r="E50" s="108" t="s">
         <v>257</v>
       </c>
-      <c r="D50" s="71" t="s">
+      <c r="F50" s="109" t="s">
         <v>261</v>
       </c>
-      <c r="E50" s="68" t="s">
+      <c r="G50" s="82" t="s">
         <v>262</v>
       </c>
-    </row>
-    <row r="51" spans="1:5" s="69" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="A51" s="64" t="s">
+      <c r="K50" s="83"/>
+      <c r="L50" s="62"/>
+      <c r="M50" s="62"/>
+      <c r="N50" s="62"/>
+      <c r="O50" s="62"/>
+      <c r="P50" s="62"/>
+      <c r="Q50" s="62"/>
+      <c r="R50" s="62"/>
+      <c r="S50" s="62"/>
+      <c r="T50" s="62"/>
+      <c r="U50" s="62"/>
+      <c r="V50" s="62"/>
+      <c r="W50" s="84"/>
+    </row>
+    <row r="51" spans="1:23" s="88" customFormat="1" x14ac:dyDescent="0.45">
+      <c r="A51" s="97" t="s">
         <v>42</v>
       </c>
-      <c r="B51" s="39" t="s">
+      <c r="B51" s="99" t="s">
         <v>182</v>
       </c>
-      <c r="C51" s="66" t="s">
+      <c r="C51" s="99"/>
+      <c r="D51" s="99"/>
+      <c r="E51" s="100" t="s">
         <v>257</v>
       </c>
-      <c r="D51" s="67" t="s">
+      <c r="F51" s="101" t="s">
         <v>261</v>
       </c>
-      <c r="E51" s="68" t="s">
+      <c r="G51" s="82" t="s">
         <v>262</v>
       </c>
-    </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A52" s="14" t="s">
+      <c r="K51" s="125"/>
+      <c r="L51" s="95"/>
+      <c r="M51" s="95"/>
+      <c r="N51" s="95"/>
+      <c r="O51" s="95"/>
+      <c r="P51" s="95"/>
+      <c r="Q51" s="95"/>
+      <c r="R51" s="95"/>
+      <c r="S51" s="95"/>
+      <c r="T51" s="95"/>
+      <c r="U51" s="95"/>
+      <c r="V51" s="95"/>
+      <c r="W51" s="96"/>
+    </row>
+    <row r="52" spans="1:23" x14ac:dyDescent="0.45">
+      <c r="A52" s="68" t="s">
         <v>43</v>
       </c>
-      <c r="B52" s="14" t="s">
+      <c r="B52" s="68" t="s">
         <v>183</v>
       </c>
-      <c r="C52" t="s">
+      <c r="C52" s="69">
+        <v>43369.178304398149</v>
+      </c>
+      <c r="D52" s="68"/>
+      <c r="E52" s="64" t="s">
         <v>257</v>
       </c>
-      <c r="D52" s="57" t="s">
+      <c r="F52" s="70" t="s">
         <v>260</v>
       </c>
-      <c r="E52" s="69" t="s">
+      <c r="G52" s="89" t="s">
+        <v>299</v>
+      </c>
+      <c r="K52" s="73">
+        <v>21.2</v>
+      </c>
+      <c r="L52" s="61">
+        <v>24.2</v>
+      </c>
+      <c r="M52" s="61">
+        <v>28.2</v>
+      </c>
+      <c r="N52" s="61">
+        <v>31.6</v>
+      </c>
+      <c r="O52" s="61"/>
+      <c r="P52" s="61"/>
+      <c r="Q52" s="61">
+        <v>22.8</v>
+      </c>
+      <c r="R52" s="61">
+        <v>26.4</v>
+      </c>
+      <c r="S52" s="61">
+        <v>29.4</v>
+      </c>
+      <c r="T52" s="61"/>
+      <c r="U52" s="61"/>
+      <c r="V52" s="61"/>
+      <c r="W52" s="70"/>
+    </row>
+    <row r="53" spans="1:23" x14ac:dyDescent="0.45">
+      <c r="A53" s="68"/>
+      <c r="B53" s="68" t="s">
+        <v>184</v>
+      </c>
+      <c r="C53" s="69">
+        <v>43369.192193287032</v>
+      </c>
+      <c r="D53" s="68"/>
+      <c r="E53" s="64" t="s">
+        <v>258</v>
+      </c>
+      <c r="F53" s="70" t="s">
+        <v>260</v>
+      </c>
+      <c r="K53" s="73">
+        <v>21.4</v>
+      </c>
+      <c r="L53" s="61">
+        <v>24.4</v>
+      </c>
+      <c r="M53" s="61">
+        <v>28.1</v>
+      </c>
+      <c r="N53" s="61">
+        <v>31.9</v>
+      </c>
+      <c r="O53" s="61"/>
+      <c r="P53" s="61"/>
+      <c r="Q53" s="61">
+        <v>23</v>
+      </c>
+      <c r="R53" s="61">
+        <v>26</v>
+      </c>
+      <c r="S53" s="61">
+        <v>30</v>
+      </c>
+      <c r="T53" s="61"/>
+      <c r="U53" s="61"/>
+      <c r="V53" s="61"/>
+      <c r="W53" s="70"/>
+    </row>
+    <row r="54" spans="1:23" x14ac:dyDescent="0.45">
+      <c r="A54" s="68"/>
+      <c r="B54" s="68" t="s">
+        <v>185</v>
+      </c>
+      <c r="C54" s="69">
+        <v>43369.219971064813</v>
+      </c>
+      <c r="D54" s="68"/>
+      <c r="E54" s="64" t="s">
+        <v>257</v>
+      </c>
+      <c r="F54" s="70" t="s">
+        <v>260</v>
+      </c>
+      <c r="G54" s="88" t="s">
         <v>268</v>
       </c>
-    </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A53" s="14"/>
-      <c r="B53" s="14" t="s">
-        <v>184</v>
-      </c>
-      <c r="C53" t="s">
-        <v>258</v>
-      </c>
-      <c r="D53" s="57" t="s">
+      <c r="K54" s="73">
+        <v>20.9</v>
+      </c>
+      <c r="L54" s="61">
+        <v>24.4</v>
+      </c>
+      <c r="M54" s="61">
+        <v>27.6</v>
+      </c>
+      <c r="N54" s="61">
+        <v>31.5</v>
+      </c>
+      <c r="O54" s="61"/>
+      <c r="P54" s="61"/>
+      <c r="Q54" s="61">
+        <v>22.7</v>
+      </c>
+      <c r="R54" s="61">
+        <v>25.9</v>
+      </c>
+      <c r="S54" s="61">
+        <v>29.7</v>
+      </c>
+      <c r="T54" s="61"/>
+      <c r="U54" s="61"/>
+      <c r="V54" s="61"/>
+      <c r="W54" s="70"/>
+    </row>
+    <row r="55" spans="1:23" x14ac:dyDescent="0.45">
+      <c r="A55" s="68"/>
+      <c r="B55" s="90" t="s">
+        <v>186</v>
+      </c>
+      <c r="C55" s="90"/>
+      <c r="D55" s="90"/>
+      <c r="E55" s="82" t="s">
+        <v>257</v>
+      </c>
+      <c r="F55" s="84" t="s">
+        <v>261</v>
+      </c>
+      <c r="G55" s="82" t="s">
+        <v>262</v>
+      </c>
+      <c r="K55" s="73"/>
+      <c r="L55" s="61"/>
+      <c r="M55" s="61"/>
+      <c r="N55" s="61"/>
+      <c r="O55" s="61"/>
+      <c r="P55" s="61"/>
+      <c r="Q55" s="61"/>
+      <c r="R55" s="61"/>
+      <c r="S55" s="61"/>
+      <c r="T55" s="61"/>
+      <c r="U55" s="61"/>
+      <c r="V55" s="61"/>
+      <c r="W55" s="70"/>
+    </row>
+    <row r="56" spans="1:23" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A56" s="63"/>
+      <c r="B56" s="110" t="s">
+        <v>187</v>
+      </c>
+      <c r="C56" s="110"/>
+      <c r="D56" s="110"/>
+      <c r="E56" s="111" t="s">
+        <v>257</v>
+      </c>
+      <c r="F56" s="112" t="s">
+        <v>261</v>
+      </c>
+      <c r="G56" s="82" t="s">
+        <v>262</v>
+      </c>
+      <c r="K56" s="115"/>
+      <c r="L56" s="63"/>
+      <c r="M56" s="63"/>
+      <c r="N56" s="63"/>
+      <c r="O56" s="63"/>
+      <c r="P56" s="63"/>
+      <c r="Q56" s="63"/>
+      <c r="R56" s="63"/>
+      <c r="S56" s="63"/>
+      <c r="T56" s="63"/>
+      <c r="U56" s="63"/>
+      <c r="V56" s="63"/>
+      <c r="W56" s="106"/>
+    </row>
+    <row r="57" spans="1:23" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
+      <c r="A57" s="64" t="s">
+        <v>38</v>
+      </c>
+      <c r="B57" s="68" t="s">
+        <v>126</v>
+      </c>
+      <c r="C57" s="69">
+        <v>42617.710376157411</v>
+      </c>
+      <c r="D57" s="69">
+        <v>42617.759739583329</v>
+      </c>
+      <c r="E57" s="64" t="s">
+        <v>257</v>
+      </c>
+      <c r="F57" s="70" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A54" s="14"/>
-      <c r="B54" s="14" t="s">
-        <v>185</v>
-      </c>
-      <c r="C54" t="s">
+      <c r="G57" s="89" t="s">
+        <v>298</v>
+      </c>
+      <c r="K57" s="73">
+        <v>20.5</v>
+      </c>
+      <c r="L57" s="61">
+        <v>24.2</v>
+      </c>
+      <c r="M57" s="61">
+        <v>27.1</v>
+      </c>
+      <c r="N57" s="61">
+        <v>30.8</v>
+      </c>
+      <c r="O57" s="61"/>
+      <c r="P57" s="61"/>
+      <c r="Q57" s="61">
+        <v>22.1</v>
+      </c>
+      <c r="R57" s="61">
+        <v>25.3</v>
+      </c>
+      <c r="S57" s="61">
+        <v>29.5</v>
+      </c>
+      <c r="T57" s="61"/>
+      <c r="U57" s="61"/>
+      <c r="V57" s="61"/>
+      <c r="W57" s="70"/>
+    </row>
+    <row r="58" spans="1:23" x14ac:dyDescent="0.45">
+      <c r="A58" s="85"/>
+      <c r="B58" s="74" t="s">
+        <v>127</v>
+      </c>
+      <c r="C58" s="75">
+        <v>42618.696718749998</v>
+      </c>
+      <c r="D58" s="75">
+        <v>42618.704241898136</v>
+      </c>
+      <c r="E58" s="85" t="s">
         <v>257</v>
       </c>
-      <c r="D54" s="57" t="s">
+      <c r="F58" s="76" t="s">
         <v>260</v>
       </c>
-      <c r="E54" s="69" t="s">
+      <c r="G58" s="64" t="s">
         <v>268</v>
       </c>
-    </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A55" s="14"/>
-      <c r="B55" s="26" t="s">
-        <v>186</v>
-      </c>
-      <c r="C55" s="68" t="s">
+      <c r="K58" s="121">
+        <v>21</v>
+      </c>
+      <c r="L58" s="85">
+        <v>24.2</v>
+      </c>
+      <c r="M58" s="85">
+        <v>28.1</v>
+      </c>
+      <c r="N58" s="85">
+        <v>31.6</v>
+      </c>
+      <c r="O58" s="85"/>
+      <c r="P58" s="85"/>
+      <c r="Q58" s="85">
+        <v>22.5</v>
+      </c>
+      <c r="R58" s="85">
+        <v>25.8</v>
+      </c>
+      <c r="S58" s="85">
+        <v>29.7</v>
+      </c>
+      <c r="T58" s="85"/>
+      <c r="U58" s="85"/>
+      <c r="V58" s="85"/>
+      <c r="W58" s="76"/>
+    </row>
+    <row r="59" spans="1:23" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A59" s="63" t="s">
+        <v>35</v>
+      </c>
+      <c r="B59" s="113" t="s">
+        <v>139</v>
+      </c>
+      <c r="C59" s="114">
+        <v>42627.17509837963</v>
+      </c>
+      <c r="D59" s="114">
+        <v>42627.183026620369</v>
+      </c>
+      <c r="E59" s="63" t="s">
         <v>257</v>
       </c>
-      <c r="D55" s="72" t="s">
-        <v>261</v>
-      </c>
-      <c r="E55" s="68" t="s">
-        <v>262</v>
-      </c>
-    </row>
-    <row r="56" spans="1:5" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A56" s="60"/>
-      <c r="B56" s="78" t="s">
-        <v>187</v>
-      </c>
-      <c r="C56" s="79" t="s">
-        <v>257</v>
-      </c>
-      <c r="D56" s="80" t="s">
-        <v>261</v>
-      </c>
-      <c r="E56" s="68" t="s">
-        <v>262</v>
-      </c>
-    </row>
-    <row r="57" spans="1:5" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="A57" t="s">
-        <v>38</v>
-      </c>
-      <c r="B57" s="14" t="s">
-        <v>126</v>
-      </c>
-      <c r="C57" t="s">
-        <v>257</v>
-      </c>
-      <c r="D57" s="57" t="s">
+      <c r="F59" s="106" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A58" s="63"/>
-      <c r="B58" s="24" t="s">
-        <v>127</v>
-      </c>
-      <c r="C58" s="63" t="s">
-        <v>257</v>
-      </c>
-      <c r="D58" s="58" t="s">
-        <v>260</v>
-      </c>
-      <c r="E58" t="s">
-        <v>268</v>
-      </c>
-    </row>
-    <row r="59" spans="1:5" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A59" s="60" t="s">
-        <v>35</v>
-      </c>
-      <c r="B59" s="33" t="s">
-        <v>139</v>
-      </c>
-      <c r="C59" s="60" t="s">
-        <v>257</v>
-      </c>
-      <c r="D59" s="77" t="s">
-        <v>260</v>
-      </c>
-      <c r="E59" t="s">
-        <v>268</v>
-      </c>
-    </row>
-    <row r="60" spans="1:5" ht="14.65" thickTop="1" x14ac:dyDescent="0.45"/>
+      <c r="G59" s="89" t="s">
+        <v>300</v>
+      </c>
+      <c r="K59" s="115"/>
+      <c r="L59" s="63"/>
+      <c r="M59" s="63"/>
+      <c r="N59" s="63"/>
+      <c r="O59" s="63"/>
+      <c r="P59" s="63"/>
+      <c r="Q59" s="63"/>
+      <c r="R59" s="63"/>
+      <c r="S59" s="63"/>
+      <c r="T59" s="63"/>
+      <c r="U59" s="63"/>
+      <c r="V59" s="63"/>
+      <c r="W59" s="106"/>
+    </row>
+    <row r="60" spans="1:23" ht="14.65" thickTop="1" x14ac:dyDescent="0.45"/>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>